<commit_message>
frontend bannder, filter fix
</commit_message>
<xml_diff>
--- a/THE (REAL) SCHEDULE.xlsx
+++ b/THE (REAL) SCHEDULE.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={b6f2e70f-835a-4c15-9b47-8562aab417fa}</author>
+    <author>tc={dbc866ff-36c2-4b34-a443-fd7ab61a53ab}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{b6f2e70f-835a-4c15-9b47-8562aab417fa}" ref="D53">
+    <comment authorId="0" xr:uid="{dbc866ff-36c2-4b34-a443-fd7ab61a53ab}" ref="D53">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -31,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="255">
-  <si>
-    <t>LAST UPDATED 3/23/26 10 AM PST</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="254">
+  <si>
+    <t>LAST UPDATED 3/24/26 3 PM PST</t>
   </si>
   <si>
     <t>Performances</t>
@@ -319,7 +319,7 @@
         <rFont val="Arial"/>
         <color rgb="FFFFFFFF"/>
       </rPr>
-      <t xml:space="preserve">8 PM-12 AM
+      <t xml:space="preserve">8:30 PM-12 AM
 </t>
     </r>
     <r>
@@ -328,7 +328,16 @@
         <i/>
         <color rgb="FFFFFFFF"/>
       </rPr>
-      <t>Bombay Bliss Beach Club</t>
+      <t xml:space="preserve">Bombay Bliss Beach Club
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t>Disco Vinyl Set starring Montel Spinoza &amp; Pierre Delecto
+Drinks and Hors D’Oeuvres</t>
     </r>
   </si>
   <si>
@@ -587,7 +596,7 @@
   <si>
     <t>Building on Questionable Foundations: An introduction to Philosophy, Art, Architecture, and Life in Bombay Beach 
 Lecture by Tao Ruspoli
-3-4 PM
+5-6 PM
 DORD, Estates 
 Philosophy Conference</t>
   </si>
@@ -680,12 +689,6 @@
 The Estates</t>
   </si>
   <si>
-    <t xml:space="preserve">Year X Opening Mixer
-6-7 PM
-Bombay Beach Yacht Club
-</t>
-  </si>
-  <si>
     <t>Birth, Life and Becoming
 by Cactus Chaos &amp; Kamau
 6-8 PM
@@ -835,7 +838,10 @@
 Queer Heaven in Bombay Beach
 7:30-9:30 PM
 The Temple to the Scientific Method
-Drag Show</t>
+Drag Show
++ Care Club
+7:30-9:30 PM
+Temple to the Scientific Method</t>
   </si>
   <si>
     <t>The Social Equilibrium Calibration Unit
@@ -876,25 +882,13 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">Care Club
-7-9:30 PM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>Temple to the Scientific Method</t>
-    </r>
+    <t>"Bombay Beach"
+by Alma Ha'rel
+7:30-9:30 PM
+Zig Zag Plaza
+Documentary Feature 
+w/ Director Alma Har'el Q&amp;A 
+BBIFF</t>
   </si>
   <si>
     <t xml:space="preserve">S.S.S.S.S's Shared Telescope Sesh
@@ -945,9 +939,9 @@
     </r>
   </si>
   <si>
-    <t>Opera &amp; Ballet
-9-10 PM
-The Opera House</t>
+    <t>Jerzy del Mar
+9-11:30 PM
+Sub Club</t>
   </si>
   <si>
     <r>
@@ -1003,21 +997,17 @@
     </r>
   </si>
   <si>
+    <t>Opera &amp; Ballet
+9:30-10:30 PM
+The Opera House</t>
+  </si>
+  <si>
     <t>LOST SOUL TRAIN 
 (Funk Musical Odyssey) 
 9:30 PM-12 AM
 The Tradewinds</t>
   </si>
   <si>
-    <t>"Bombay Beach"
-by Alma Ha'rel
-10 PM-12 
-Henderson Hall
-Documentary Feature 
-w/ Director Q&amp;A 
-BBIFF</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
@@ -1049,11 +1039,6 @@
 RaphaLots
 </t>
     </r>
-  </si>
-  <si>
-    <t>Heidi and Love Fingers
-10 PM-2 AM
-Sub Club</t>
   </si>
   <si>
     <t>The Last Canter
@@ -1087,6 +1072,11 @@
     </r>
   </si>
   <si>
+    <t>Flamenco Performance
+11 PM-12 AM
+Zig Zag Plaza</t>
+  </si>
+  <si>
     <t>Late Night Bliss
 11 PM-3 AM
 Bombay Bliss Beach Club</t>
@@ -1120,12 +1110,12 @@
     </r>
   </si>
   <si>
+    <t>Heidi Lawden &amp; LoveFingers (B2B)
+11:30 PM-3 AM
+Sub Club</t>
+  </si>
+  <si>
     <t>SATURDAY</t>
-  </si>
-  <si>
-    <t>Flamenco Performance
-12-1 AM
-Zig Zag Plaza</t>
   </si>
   <si>
     <t>Globalschism
@@ -3757,7 +3747,7 @@
     <xf borderId="4" fillId="11" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="15" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="20" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -3778,6 +3768,9 @@
     <xf borderId="3" fillId="0" fontId="14" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="10" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="4" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -3793,13 +3786,16 @@
     <xf borderId="0" fillId="15" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="2" fillId="2" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="11" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="22" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -3814,9 +3810,6 @@
     <xf borderId="5" fillId="15" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="4" fillId="9" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -3911,9 +3904,6 @@
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="15" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -3997,7 +3987,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Dane Sandborg" id="{d7f21a1f-7073-41c4-a3b9-cda45052e0bb}" providerId="google-sheets"/>
+  <x18tc:person displayName="Dane Sandborg" id="{86379b4e-de9c-4987-864f-db4cceedcc00}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -4197,7 +4187,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D53" dT="2026-03-23T19:38:09.00" personId="{d7f21a1f-7073-41c4-a3b9-cda45052e0bb}" id="{b6f2e70f-835a-4c15-9b47-8562aab417fa}" done="0">
+  <x18tc:threadedComment ref="D53" dT="2026-03-23T19:38:09.00" personId="{86379b4e-de9c-4987-864f-db4cceedcc00}" id="{dbc866ff-36c2-4b34-a443-fd7ab61a53ab}" done="0">
     <x18tc:text xml:space="preserve">The lost soul train</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -5103,26 +5093,24 @@
         <v>0.75</v>
       </c>
       <c r="C77" s="40"/>
-      <c r="D77" s="91" t="s">
-        <v>60</v>
-      </c>
+      <c r="D77" s="91"/>
       <c r="E77" s="17"/>
       <c r="F77" s="40"/>
       <c r="G77" s="40"/>
       <c r="H77" s="76"/>
       <c r="I77" s="92" t="s">
+        <v>60</v>
+      </c>
+      <c r="J77" s="93" t="s">
         <v>61</v>
-      </c>
-      <c r="J77" s="93" t="s">
-        <v>62</v>
       </c>
       <c r="K77" s="40"/>
       <c r="L77" s="64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N77" s="40"/>
       <c r="O77" s="33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P77" s="40"/>
     </row>
@@ -5139,7 +5127,7 @@
       <c r="J78" s="40"/>
       <c r="K78" s="40"/>
       <c r="L78" s="30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N78" s="40"/>
       <c r="O78" s="40"/>
@@ -5152,24 +5140,24 @@
       </c>
       <c r="C79" s="40"/>
       <c r="D79" s="56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E79" s="17"/>
       <c r="F79" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="G79" s="95" t="s">
         <v>67</v>
       </c>
-      <c r="G79" s="95" t="s">
+      <c r="H79" s="96" t="s">
         <v>68</v>
-      </c>
-      <c r="H79" s="96" t="s">
-        <v>69</v>
       </c>
       <c r="I79" s="40"/>
       <c r="J79" s="40"/>
       <c r="K79" s="41"/>
       <c r="L79" s="40"/>
       <c r="M79" s="56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N79" s="40"/>
       <c r="O79" s="40"/>
@@ -5181,14 +5169,14 @@
       <c r="C80" s="40"/>
       <c r="D80" s="40"/>
       <c r="E80" s="58" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F80" s="41"/>
       <c r="H80" s="40"/>
       <c r="I80" s="41"/>
       <c r="J80" s="41"/>
       <c r="K80" s="30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L80" s="40"/>
       <c r="M80" s="40"/>
@@ -5202,28 +5190,28 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C81" s="80" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D81" s="40"/>
       <c r="E81" s="40"/>
-      <c r="F81" s="30" t="s">
-        <v>74</v>
+      <c r="F81" s="98" t="s">
+        <v>73</v>
       </c>
       <c r="H81" s="40"/>
       <c r="I81" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="J81" s="99" t="s">
         <v>75</v>
       </c>
-      <c r="J81" s="98" t="s">
+      <c r="K81" s="30" t="s">
         <v>76</v>
-      </c>
-      <c r="K81" s="30" t="s">
-        <v>77</v>
       </c>
       <c r="L81" s="40"/>
       <c r="M81" s="40"/>
       <c r="N81" s="40"/>
       <c r="O81" s="56" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P81" s="40"/>
     </row>
@@ -5250,38 +5238,38 @@
         <v>0.875</v>
       </c>
       <c r="C83" s="41"/>
-      <c r="D83" s="58" t="s">
+      <c r="E83" s="95" t="s">
+        <v>78</v>
+      </c>
+      <c r="F83" s="40"/>
+      <c r="G83" s="100" t="s">
         <v>79</v>
       </c>
-      <c r="E83" s="41"/>
-      <c r="F83" s="40"/>
-      <c r="G83" s="99" t="s">
+      <c r="H83" s="30" t="s">
         <v>80</v>
-      </c>
-      <c r="H83" s="30" t="s">
-        <v>81</v>
       </c>
       <c r="I83" s="45"/>
       <c r="J83" s="40"/>
       <c r="K83" s="40"/>
       <c r="L83" s="40"/>
-      <c r="M83" s="100" t="s">
-        <v>82</v>
+      <c r="M83" s="101" t="s">
+        <v>81</v>
       </c>
       <c r="N83" s="40"/>
       <c r="O83" s="40"/>
       <c r="P83" s="40"/>
     </row>
-    <row r="84" ht="85.5" customHeight="1">
+    <row r="84" ht="73.5" customHeight="1">
       <c r="A84" s="21"/>
       <c r="B84" s="17"/>
       <c r="C84" s="18"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="31"/>
-      <c r="F84" s="41"/>
+      <c r="D84" s="58" t="s">
+        <v>82</v>
+      </c>
+      <c r="F84" s="40"/>
       <c r="G84" s="40"/>
       <c r="H84" s="41"/>
-      <c r="I84" s="101" t="s">
+      <c r="I84" s="102" t="s">
         <v>83</v>
       </c>
       <c r="J84" s="41"/>
@@ -5292,41 +5280,36 @@
       <c r="O84" s="41"/>
       <c r="P84" s="40"/>
     </row>
-    <row r="85" ht="52.5" customHeight="1">
+    <row r="85" ht="42.0" customHeight="1">
       <c r="A85" s="21"/>
       <c r="B85" s="97">
         <v>0.9166666666666666</v>
       </c>
-      <c r="C85" s="102"/>
-      <c r="D85" s="103" t="s">
+      <c r="C85" s="103"/>
+      <c r="D85" s="38"/>
+      <c r="F85" s="104" t="s">
         <v>84</v>
       </c>
-      <c r="F85" s="104" t="s">
-        <v>85</v>
-      </c>
       <c r="G85" s="40"/>
-      <c r="H85" s="95" t="s">
-        <v>86</v>
-      </c>
+      <c r="H85" s="105"/>
       <c r="I85" s="40"/>
       <c r="J85" s="56" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="K85" s="40"/>
-      <c r="L85" s="105" t="s">
-        <v>88</v>
+      <c r="L85" s="106" t="s">
+        <v>86</v>
       </c>
       <c r="M85" s="40"/>
       <c r="N85" s="40"/>
-      <c r="O85" s="98" t="s">
-        <v>76</v>
+      <c r="O85" s="99" t="s">
+        <v>75</v>
       </c>
       <c r="P85" s="40"/>
     </row>
-    <row r="86" ht="30.0" customHeight="1">
+    <row r="86" ht="24.75" customHeight="1">
       <c r="A86" s="21"/>
       <c r="B86" s="17"/>
-      <c r="D86" s="40"/>
       <c r="F86" s="17"/>
       <c r="G86" s="40"/>
       <c r="I86" s="40"/>
@@ -5342,17 +5325,19 @@
       <c r="B87" s="97">
         <v>0.9583333333333334</v>
       </c>
-      <c r="D87" s="40"/>
+      <c r="D87" s="107" t="s">
+        <v>87</v>
+      </c>
       <c r="F87" s="17"/>
       <c r="G87" s="40"/>
       <c r="I87" s="40"/>
       <c r="J87" s="40"/>
       <c r="K87" s="40"/>
       <c r="M87" s="95" t="s">
+        <v>88</v>
+      </c>
+      <c r="N87" s="95" t="s">
         <v>89</v>
-      </c>
-      <c r="N87" s="95" t="s">
-        <v>90</v>
       </c>
       <c r="O87" s="40"/>
       <c r="P87" s="40"/>
@@ -5360,7 +5345,9 @@
     <row r="88" ht="87.0" customHeight="1">
       <c r="A88" s="21"/>
       <c r="B88" s="66"/>
-      <c r="D88" s="41"/>
+      <c r="E88" s="95" t="s">
+        <v>90</v>
+      </c>
       <c r="F88" s="66"/>
       <c r="G88" s="41"/>
       <c r="I88" s="41"/>
@@ -5371,62 +5358,60 @@
     </row>
     <row r="89">
       <c r="A89" s="21"/>
-      <c r="B89" s="106" t="s">
+      <c r="B89" s="108" t="s">
         <v>91</v>
       </c>
-      <c r="C89" s="107"/>
-      <c r="E89" s="108"/>
-      <c r="F89" s="108"/>
-      <c r="G89" s="108"/>
-      <c r="H89" s="108"/>
-      <c r="I89" s="108"/>
-      <c r="J89" s="108"/>
-      <c r="K89" s="108"/>
-      <c r="L89" s="108"/>
-      <c r="M89" s="108"/>
-      <c r="N89" s="108"/>
-      <c r="O89" s="108"/>
-      <c r="P89" s="108"/>
+      <c r="C89" s="109"/>
+      <c r="E89" s="110"/>
+      <c r="F89" s="110"/>
+      <c r="G89" s="110"/>
+      <c r="H89" s="110"/>
+      <c r="I89" s="110"/>
+      <c r="J89" s="110"/>
+      <c r="K89" s="110"/>
+      <c r="L89" s="110"/>
+      <c r="M89" s="110"/>
+      <c r="N89" s="110"/>
+      <c r="O89" s="110"/>
+      <c r="P89" s="110"/>
     </row>
     <row r="90" ht="77.25" customHeight="1">
       <c r="A90" s="21"/>
       <c r="B90" s="79">
         <v>1.0</v>
       </c>
-      <c r="C90" s="109"/>
-      <c r="D90" s="110" t="s">
+      <c r="C90" s="111"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="95" t="s">
+        <v>90</v>
+      </c>
+      <c r="F90" s="95" t="s">
         <v>92</v>
       </c>
-      <c r="E90" s="38"/>
-      <c r="F90" s="95" t="s">
+      <c r="G90" s="100" t="s">
         <v>93</v>
       </c>
-      <c r="G90" s="99" t="s">
+      <c r="H90" s="105"/>
+      <c r="I90" s="95" t="s">
         <v>94</v>
       </c>
-      <c r="H90" s="95" t="s">
-        <v>86</v>
-      </c>
-      <c r="I90" s="95" t="s">
+      <c r="J90" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="K90" s="100" t="s">
         <v>95</v>
       </c>
-      <c r="J90" s="56" t="s">
-        <v>87</v>
-      </c>
-      <c r="K90" s="99" t="s">
+      <c r="L90" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="M90" s="95" t="s">
+        <v>88</v>
+      </c>
+      <c r="N90" s="95" t="s">
         <v>96</v>
       </c>
-      <c r="L90" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="M90" s="95" t="s">
-        <v>89</v>
-      </c>
-      <c r="N90" s="95" t="s">
-        <v>97</v>
-      </c>
-      <c r="O90" s="98" t="s">
-        <v>76</v>
+      <c r="O90" s="99" t="s">
+        <v>75</v>
       </c>
       <c r="P90" s="90" t="s">
         <v>59</v>
@@ -5436,8 +5421,8 @@
       <c r="A91" s="21"/>
       <c r="B91" s="40"/>
       <c r="C91" s="40"/>
-      <c r="E91" s="111" t="s">
-        <v>98</v>
+      <c r="D91" s="112" t="s">
+        <v>97</v>
       </c>
       <c r="G91" s="40"/>
       <c r="J91" s="40"/>
@@ -5452,8 +5437,7 @@
         <v>0.041666666666666664</v>
       </c>
       <c r="C92" s="40"/>
-      <c r="D92" s="31"/>
-      <c r="E92" s="40"/>
+      <c r="D92" s="40"/>
       <c r="G92" s="40"/>
       <c r="J92" s="40"/>
       <c r="K92" s="40"/>
@@ -5465,7 +5449,7 @@
       <c r="A93" s="21"/>
       <c r="B93" s="79"/>
       <c r="C93" s="40"/>
-      <c r="E93" s="40"/>
+      <c r="D93" s="40"/>
       <c r="G93" s="41"/>
       <c r="J93" s="41"/>
       <c r="K93" s="41"/>
@@ -5479,22 +5463,21 @@
         <v>0.08333333333333333</v>
       </c>
       <c r="C94" s="40"/>
-      <c r="E94" s="41"/>
+      <c r="D94" s="41"/>
       <c r="F94" s="39"/>
       <c r="G94" s="31"/>
-      <c r="H94" s="31"/>
       <c r="I94" s="38"/>
       <c r="J94" s="38"/>
-      <c r="K94" s="112"/>
+      <c r="K94" s="113"/>
       <c r="L94" s="39"/>
-      <c r="O94" s="112"/>
+      <c r="O94" s="113"/>
       <c r="P94" s="40"/>
     </row>
     <row r="95" ht="21.0" customHeight="1">
       <c r="A95" s="21"/>
       <c r="B95" s="79"/>
       <c r="C95" s="40"/>
-      <c r="E95" s="113"/>
+      <c r="D95" s="38"/>
       <c r="K95" s="40"/>
       <c r="M95" s="95"/>
       <c r="N95" s="95"/>
@@ -5507,8 +5490,9 @@
         <v>0.125</v>
       </c>
       <c r="C96" s="40"/>
+      <c r="E96" s="114"/>
       <c r="K96" s="40"/>
-      <c r="M96" s="114"/>
+      <c r="M96" s="115"/>
       <c r="N96" s="31"/>
       <c r="O96" s="40"/>
       <c r="P96" s="40"/>
@@ -5564,18 +5548,18 @@
       </c>
       <c r="K101" s="40"/>
       <c r="O101" s="37" t="s">
-        <v>99</v>
-      </c>
-      <c r="P101" s="115"/>
-    </row>
-    <row r="102" ht="92.25" customHeight="1">
+        <v>98</v>
+      </c>
+      <c r="P101" s="116"/>
+    </row>
+    <row r="102" ht="111.0" customHeight="1">
       <c r="A102" s="21"/>
       <c r="B102" s="79">
         <v>0.375</v>
       </c>
       <c r="C102" s="40"/>
       <c r="D102" s="64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J102" s="40"/>
       <c r="K102" s="40"/>
@@ -5589,16 +5573,16 @@
       </c>
       <c r="C103" s="40"/>
       <c r="D103" s="83" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E103" s="64" t="s">
         <v>40</v>
       </c>
       <c r="F103" s="87" t="s">
+        <v>101</v>
+      </c>
+      <c r="H103" s="30" t="s">
         <v>102</v>
-      </c>
-      <c r="H103" s="30" t="s">
-        <v>103</v>
       </c>
       <c r="J103" s="40"/>
       <c r="K103" s="40"/>
@@ -5610,8 +5594,8 @@
       <c r="B104" s="40"/>
       <c r="C104" s="40"/>
       <c r="D104" s="40"/>
-      <c r="E104" s="116" t="s">
-        <v>104</v>
+      <c r="E104" s="117" t="s">
+        <v>103</v>
       </c>
       <c r="F104" s="41"/>
       <c r="G104" s="69"/>
@@ -5628,25 +5612,25 @@
       </c>
       <c r="C105" s="40"/>
       <c r="D105" s="83" t="s">
+        <v>104</v>
+      </c>
+      <c r="E105" s="38"/>
+      <c r="F105" s="118" t="s">
         <v>105</v>
       </c>
-      <c r="E105" s="38"/>
-      <c r="F105" s="117" t="s">
+      <c r="G105" s="99" t="s">
         <v>106</v>
-      </c>
-      <c r="G105" s="98" t="s">
-        <v>107</v>
       </c>
       <c r="H105" s="30" t="s">
         <v>42</v>
       </c>
       <c r="I105" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J105" s="40"/>
       <c r="K105" s="40"/>
       <c r="L105" s="56" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O105" s="40"/>
       <c r="P105" s="40"/>
@@ -5656,8 +5640,8 @@
       <c r="B106" s="40"/>
       <c r="C106" s="40"/>
       <c r="D106" s="40"/>
-      <c r="E106" s="118" t="s">
-        <v>110</v>
+      <c r="E106" s="119" t="s">
+        <v>109</v>
       </c>
       <c r="F106" s="41"/>
       <c r="G106" s="40"/>
@@ -5676,18 +5660,18 @@
       </c>
       <c r="C107" s="40"/>
       <c r="D107" s="83" t="s">
+        <v>110</v>
+      </c>
+      <c r="E107" s="41"/>
+      <c r="F107" s="120" t="s">
         <v>111</v>
-      </c>
-      <c r="E107" s="41"/>
-      <c r="F107" s="119" t="s">
-        <v>112</v>
       </c>
       <c r="G107" s="40"/>
       <c r="H107" s="40"/>
       <c r="I107" s="40"/>
       <c r="J107" s="40"/>
       <c r="K107" s="56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L107" s="40"/>
       <c r="O107" s="40"/>
@@ -5696,7 +5680,7 @@
     <row r="108" ht="52.5" customHeight="1">
       <c r="A108" s="21"/>
       <c r="B108" s="40"/>
-      <c r="C108" s="109"/>
+      <c r="C108" s="111"/>
       <c r="D108" s="40"/>
       <c r="E108" s="31"/>
       <c r="F108" s="40"/>
@@ -5715,18 +5699,18 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="C109" s="80" t="s">
+        <v>113</v>
+      </c>
+      <c r="D109" s="83" t="s">
         <v>114</v>
       </c>
-      <c r="D109" s="83" t="s">
+      <c r="E109" s="120" t="s">
         <v>115</v>
-      </c>
-      <c r="E109" s="119" t="s">
-        <v>116</v>
       </c>
       <c r="F109" s="40"/>
       <c r="G109" s="31"/>
       <c r="H109" s="30" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I109" s="40"/>
       <c r="J109" s="40"/>
@@ -5743,7 +5727,7 @@
       <c r="E110" s="40"/>
       <c r="F110" s="40"/>
       <c r="G110" s="30" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H110" s="41"/>
       <c r="I110" s="40"/>
@@ -5759,8 +5743,8 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C111" s="40"/>
-      <c r="D111" s="120" t="s">
-        <v>119</v>
+      <c r="D111" s="121" t="s">
+        <v>118</v>
       </c>
       <c r="E111" s="40"/>
       <c r="F111" s="40"/>
@@ -5768,12 +5752,12 @@
       <c r="H111" s="38"/>
       <c r="I111" s="40"/>
       <c r="J111" s="30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K111" s="40"/>
       <c r="L111" s="40"/>
       <c r="M111" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O111" s="40"/>
       <c r="P111" s="40"/>
@@ -5799,20 +5783,20 @@
       <c r="B113" s="94">
         <v>0.625</v>
       </c>
-      <c r="C113" s="121"/>
+      <c r="C113" s="122"/>
       <c r="D113" s="83" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E113" s="41"/>
       <c r="F113" s="40"/>
       <c r="G113" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="H113" s="123" t="s">
         <v>123</v>
       </c>
-      <c r="H113" s="122" t="s">
+      <c r="I113" s="118" t="s">
         <v>124</v>
-      </c>
-      <c r="I113" s="117" t="s">
-        <v>125</v>
       </c>
       <c r="J113" s="40"/>
       <c r="K113" s="40"/>
@@ -5828,20 +5812,20 @@
       </c>
       <c r="C114" s="17"/>
       <c r="D114" s="83" t="s">
+        <v>125</v>
+      </c>
+      <c r="E114" s="56" t="s">
         <v>126</v>
       </c>
-      <c r="E114" s="56" t="s">
+      <c r="F114" s="30" t="s">
         <v>127</v>
-      </c>
-      <c r="F114" s="30" t="s">
-        <v>128</v>
       </c>
       <c r="G114" s="40"/>
       <c r="H114" s="40"/>
       <c r="I114" s="40"/>
       <c r="J114" s="40"/>
       <c r="K114" s="30" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L114" s="40"/>
       <c r="M114" s="41"/>
@@ -5861,7 +5845,7 @@
       <c r="J115" s="41"/>
       <c r="K115" s="40"/>
       <c r="L115" s="40"/>
-      <c r="M115" s="114"/>
+      <c r="M115" s="115"/>
       <c r="O115" s="40"/>
       <c r="P115" s="40"/>
     </row>
@@ -5872,7 +5856,7 @@
       </c>
       <c r="C116" s="17"/>
       <c r="D116" s="30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E116" s="41"/>
       <c r="F116" s="40"/>
@@ -5880,14 +5864,14 @@
         <v>54</v>
       </c>
       <c r="H116" s="41"/>
-      <c r="I116" s="117" t="s">
-        <v>131</v>
+      <c r="I116" s="118" t="s">
+        <v>130</v>
       </c>
       <c r="J116" s="38"/>
       <c r="K116" s="40"/>
       <c r="L116" s="40"/>
       <c r="N116" s="56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O116" s="40"/>
       <c r="P116" s="40"/>
@@ -5898,7 +5882,7 @@
       <c r="C117" s="17"/>
       <c r="D117" s="41"/>
       <c r="E117" s="64" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F117" s="40"/>
       <c r="G117" s="40"/>
@@ -5916,32 +5900,32 @@
         <v>0.75</v>
       </c>
       <c r="C118" s="17"/>
-      <c r="D118" s="123" t="s">
+      <c r="D118" s="124" t="s">
+        <v>133</v>
+      </c>
+      <c r="E118" s="125" t="s">
         <v>134</v>
-      </c>
-      <c r="E118" s="124" t="s">
-        <v>135</v>
       </c>
       <c r="F118" s="40"/>
       <c r="G118" s="40"/>
       <c r="H118" s="56" t="s">
+        <v>135</v>
+      </c>
+      <c r="I118" s="40"/>
+      <c r="J118" s="126" t="s">
         <v>136</v>
       </c>
-      <c r="I118" s="40"/>
-      <c r="J118" s="125" t="s">
-        <v>137</v>
-      </c>
-      <c r="K118" s="112"/>
+      <c r="K118" s="113"/>
       <c r="L118" s="30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M118" s="33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N118" s="40"/>
       <c r="O118" s="40"/>
-      <c r="P118" s="126" t="s">
-        <v>138</v>
+      <c r="P118" s="127" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="119" ht="51.0" customHeight="1">
@@ -5969,27 +5953,27 @@
       </c>
       <c r="C120" s="17"/>
       <c r="D120" s="83" t="s">
+        <v>138</v>
+      </c>
+      <c r="E120" s="30" t="s">
         <v>139</v>
-      </c>
-      <c r="E120" s="30" t="s">
-        <v>140</v>
       </c>
       <c r="F120" s="40"/>
       <c r="G120" s="95" t="s">
+        <v>140</v>
+      </c>
+      <c r="H120" s="56" t="s">
         <v>141</v>
       </c>
-      <c r="H120" s="56" t="s">
+      <c r="I120" s="56" t="s">
         <v>142</v>
-      </c>
-      <c r="I120" s="56" t="s">
-        <v>143</v>
       </c>
       <c r="J120" s="40"/>
       <c r="K120" s="40"/>
       <c r="L120" s="40"/>
       <c r="M120" s="40"/>
       <c r="N120" s="56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O120" s="40"/>
       <c r="P120" s="40"/>
@@ -5999,8 +5983,8 @@
       <c r="B121" s="40"/>
       <c r="C121" s="17"/>
       <c r="D121" s="40"/>
-      <c r="E121" s="124" t="s">
-        <v>144</v>
+      <c r="E121" s="125" t="s">
+        <v>143</v>
       </c>
       <c r="F121" s="40"/>
       <c r="H121" s="41"/>
@@ -6019,35 +6003,35 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C122" s="80" t="s">
+        <v>144</v>
+      </c>
+      <c r="D122" s="40"/>
+      <c r="E122" s="125" t="s">
         <v>145</v>
       </c>
-      <c r="D122" s="40"/>
-      <c r="E122" s="124" t="s">
+      <c r="F122" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="H122" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="F122" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="H122" s="58" t="s">
+      <c r="I122" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="I122" s="46" t="s">
+      <c r="J122" s="126" t="s">
         <v>148</v>
       </c>
-      <c r="J122" s="125" t="s">
+      <c r="K122" s="118" t="s">
         <v>149</v>
       </c>
-      <c r="K122" s="117" t="s">
+      <c r="L122" s="56" t="s">
         <v>150</v>
       </c>
-      <c r="L122" s="56" t="s">
+      <c r="M122" s="126" t="s">
         <v>151</v>
       </c>
-      <c r="M122" s="125" t="s">
+      <c r="N122" s="56" t="s">
         <v>152</v>
-      </c>
-      <c r="N122" s="56" t="s">
-        <v>153</v>
       </c>
       <c r="O122" s="40"/>
       <c r="P122" s="40"/>
@@ -6060,7 +6044,7 @@
       <c r="E123" s="40"/>
       <c r="F123" s="40"/>
       <c r="G123" s="87" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H123" s="40"/>
       <c r="I123" s="41"/>
@@ -6078,28 +6062,28 @@
         <v>0.875</v>
       </c>
       <c r="C124" s="41"/>
-      <c r="D124" s="120" t="s">
+      <c r="D124" s="121" t="s">
+        <v>154</v>
+      </c>
+      <c r="E124" s="125" t="s">
         <v>155</v>
       </c>
-      <c r="E124" s="124" t="s">
-        <v>156</v>
-      </c>
       <c r="F124" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G124" s="41"/>
       <c r="H124" s="41"/>
       <c r="I124" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="J124" s="30" t="s">
         <v>157</v>
-      </c>
-      <c r="J124" s="30" t="s">
-        <v>158</v>
       </c>
       <c r="K124" s="40"/>
       <c r="L124" s="40"/>
       <c r="M124" s="38"/>
       <c r="N124" s="89" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O124" s="40"/>
       <c r="P124" s="40"/>
@@ -6112,7 +6096,7 @@
       <c r="E125" s="41"/>
       <c r="F125" s="40"/>
       <c r="G125" s="31"/>
-      <c r="H125" s="127"/>
+      <c r="H125" s="128"/>
       <c r="I125" s="40"/>
       <c r="J125" s="41"/>
       <c r="K125" s="41"/>
@@ -6126,35 +6110,35 @@
       <c r="B126" s="79">
         <v>0.9166666666666666</v>
       </c>
-      <c r="C126" s="128"/>
+      <c r="C126" s="129"/>
       <c r="D126" s="31"/>
-      <c r="E126" s="129" t="s">
+      <c r="E126" s="130" t="s">
+        <v>159</v>
+      </c>
+      <c r="F126" s="131" t="s">
         <v>160</v>
       </c>
-      <c r="F126" s="130" t="s">
+      <c r="G126" s="99" t="s">
         <v>161</v>
       </c>
-      <c r="G126" s="98" t="s">
+      <c r="H126" s="132" t="s">
         <v>162</v>
       </c>
-      <c r="H126" s="131" t="s">
+      <c r="I126" s="95" t="s">
         <v>163</v>
       </c>
-      <c r="I126" s="95" t="s">
+      <c r="J126" s="106" t="s">
         <v>164</v>
       </c>
-      <c r="J126" s="105" t="s">
+      <c r="K126" s="126" t="s">
         <v>165</v>
       </c>
-      <c r="K126" s="125" t="s">
+      <c r="L126" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="N126" s="40"/>
+      <c r="O126" s="106" t="s">
         <v>166</v>
-      </c>
-      <c r="L126" s="56" t="s">
-        <v>87</v>
-      </c>
-      <c r="N126" s="40"/>
-      <c r="O126" s="105" t="s">
-        <v>167</v>
       </c>
       <c r="P126" s="40"/>
     </row>
@@ -6177,26 +6161,26 @@
         <v>0.9583333333333334</v>
       </c>
       <c r="C128" s="17"/>
-      <c r="D128" s="132" t="s">
+      <c r="D128" s="133" t="s">
+        <v>167</v>
+      </c>
+      <c r="E128" s="106" t="s">
         <v>168</v>
       </c>
-      <c r="E128" s="105" t="s">
+      <c r="F128" s="40"/>
+      <c r="G128" s="100" t="s">
         <v>169</v>
       </c>
-      <c r="F128" s="40"/>
-      <c r="G128" s="99" t="s">
+      <c r="H128" s="40"/>
+      <c r="I128" s="134" t="s">
         <v>170</v>
       </c>
-      <c r="H128" s="40"/>
-      <c r="I128" s="133" t="s">
+      <c r="K128" s="126" t="s">
         <v>171</v>
       </c>
-      <c r="K128" s="125" t="s">
+      <c r="L128" s="40"/>
+      <c r="M128" s="135" t="s">
         <v>172</v>
-      </c>
-      <c r="L128" s="40"/>
-      <c r="M128" s="134" t="s">
-        <v>173</v>
       </c>
       <c r="N128" s="40"/>
       <c r="P128" s="40"/>
@@ -6210,7 +6194,7 @@
       <c r="G129" s="41"/>
       <c r="H129" s="41"/>
       <c r="I129" s="95" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K129" s="41"/>
       <c r="L129" s="41"/>
@@ -6220,65 +6204,65 @@
     </row>
     <row r="130">
       <c r="A130" s="21"/>
-      <c r="B130" s="135" t="s">
+      <c r="B130" s="136" t="s">
         <v>11</v>
       </c>
-      <c r="C130" s="136"/>
-      <c r="E130" s="137"/>
-      <c r="F130" s="137"/>
-      <c r="G130" s="137"/>
-      <c r="H130" s="137"/>
-      <c r="I130" s="138"/>
+      <c r="C130" s="137"/>
+      <c r="E130" s="138"/>
+      <c r="F130" s="138"/>
+      <c r="G130" s="138"/>
+      <c r="H130" s="138"/>
+      <c r="I130" s="139"/>
       <c r="J130" s="69"/>
       <c r="K130" s="88"/>
-      <c r="L130" s="139"/>
-      <c r="M130" s="139"/>
-      <c r="N130" s="140"/>
-      <c r="O130" s="141"/>
-      <c r="P130" s="141"/>
+      <c r="L130" s="140"/>
+      <c r="M130" s="140"/>
+      <c r="N130" s="141"/>
+      <c r="O130" s="142"/>
+      <c r="P130" s="142"/>
     </row>
     <row r="131" ht="30.0" customHeight="1">
       <c r="A131" s="21"/>
       <c r="B131" s="79">
         <v>1.0</v>
       </c>
-      <c r="C131" s="128"/>
-      <c r="D131" s="132" t="s">
+      <c r="C131" s="129"/>
+      <c r="D131" s="133" t="s">
+        <v>173</v>
+      </c>
+      <c r="E131" s="106" t="s">
+        <v>168</v>
+      </c>
+      <c r="F131" s="95" t="s">
+        <v>92</v>
+      </c>
+      <c r="G131" s="100" t="s">
         <v>174</v>
       </c>
-      <c r="E131" s="105" t="s">
-        <v>169</v>
-      </c>
-      <c r="F131" s="95" t="s">
-        <v>93</v>
-      </c>
-      <c r="G131" s="99" t="s">
+      <c r="H131" s="132" t="s">
+        <v>162</v>
+      </c>
+      <c r="I131" s="95" t="s">
         <v>175</v>
       </c>
-      <c r="H131" s="131" t="s">
-        <v>163</v>
-      </c>
-      <c r="I131" s="95" t="s">
+      <c r="J131" s="106" t="s">
+        <v>164</v>
+      </c>
+      <c r="K131" s="126" t="s">
         <v>176</v>
       </c>
-      <c r="J131" s="105" t="s">
-        <v>165</v>
-      </c>
-      <c r="K131" s="125" t="s">
-        <v>177</v>
-      </c>
       <c r="L131" s="56" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M131" s="38"/>
       <c r="N131" s="89" t="s">
+        <v>177</v>
+      </c>
+      <c r="O131" s="106" t="s">
         <v>178</v>
       </c>
-      <c r="O131" s="105" t="s">
+      <c r="P131" s="127" t="s">
         <v>179</v>
-      </c>
-      <c r="P131" s="126" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="132" ht="48.75" customHeight="1">
@@ -6300,13 +6284,13 @@
       </c>
       <c r="C133" s="17"/>
       <c r="D133" s="41"/>
-      <c r="E133" s="105" t="s">
-        <v>181</v>
+      <c r="E133" s="106" t="s">
+        <v>180</v>
       </c>
       <c r="G133" s="40"/>
       <c r="H133" s="41"/>
-      <c r="K133" s="99" t="s">
-        <v>182</v>
+      <c r="K133" s="100" t="s">
+        <v>181</v>
       </c>
       <c r="L133" s="41"/>
       <c r="N133" s="40"/>
@@ -6326,7 +6310,7 @@
       <c r="K134" s="40"/>
       <c r="L134" s="39"/>
       <c r="N134" s="40"/>
-      <c r="O134" s="142"/>
+      <c r="O134" s="143"/>
       <c r="P134" s="40"/>
     </row>
     <row r="135" ht="31.5" customHeight="1">
@@ -6335,8 +6319,8 @@
         <v>0.125</v>
       </c>
       <c r="C135" s="17"/>
-      <c r="E135" s="105" t="s">
-        <v>183</v>
+      <c r="E135" s="106" t="s">
+        <v>182</v>
       </c>
       <c r="G135" s="31"/>
       <c r="I135" s="31"/>
@@ -6361,10 +6345,10 @@
       </c>
       <c r="C137" s="17"/>
       <c r="E137" s="95" t="s">
+        <v>183</v>
+      </c>
+      <c r="H137" s="30" t="s">
         <v>184</v>
-      </c>
-      <c r="H137" s="30" t="s">
-        <v>185</v>
       </c>
       <c r="K137" s="39"/>
       <c r="N137" s="40"/>
@@ -6377,7 +6361,7 @@
       </c>
       <c r="C138" s="17"/>
       <c r="D138" s="30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H138" s="40"/>
       <c r="N138" s="41"/>
@@ -6391,7 +6375,7 @@
       <c r="C139" s="17"/>
       <c r="D139" s="40"/>
       <c r="E139" s="95" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H139" s="40"/>
       <c r="N139" s="39"/>
@@ -6405,7 +6389,7 @@
       <c r="C140" s="17"/>
       <c r="D140" s="40"/>
       <c r="G140" s="37" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H140" s="40"/>
     </row>
@@ -6416,11 +6400,11 @@
       </c>
       <c r="C141" s="17"/>
       <c r="D141" s="41"/>
-      <c r="E141" s="143"/>
+      <c r="E141" s="105"/>
       <c r="G141" s="40"/>
       <c r="H141" s="40"/>
       <c r="I141" s="30" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="142" ht="61.5" customHeight="1">
@@ -6429,10 +6413,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C142" s="80" t="s">
+        <v>189</v>
+      </c>
+      <c r="D142" s="30" t="s">
         <v>190</v>
-      </c>
-      <c r="D142" s="30" t="s">
-        <v>191</v>
       </c>
       <c r="F142" s="64" t="s">
         <v>40</v>
@@ -6458,10 +6442,10 @@
       </c>
       <c r="C144" s="41"/>
       <c r="D144" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="F144" s="56" t="s">
         <v>192</v>
-      </c>
-      <c r="F144" s="56" t="s">
-        <v>193</v>
       </c>
       <c r="G144" s="40"/>
       <c r="H144" s="41"/>
@@ -6473,13 +6457,13 @@
         <v>0.5</v>
       </c>
       <c r="C145" s="144" t="s">
+        <v>193</v>
+      </c>
+      <c r="D145" s="64" t="s">
         <v>194</v>
       </c>
-      <c r="D145" s="64" t="s">
+      <c r="E145" s="120" t="s">
         <v>195</v>
-      </c>
-      <c r="E145" s="119" t="s">
-        <v>196</v>
       </c>
       <c r="F145" s="40"/>
       <c r="G145" s="40"/>
@@ -6492,7 +6476,7 @@
       </c>
       <c r="C146" s="66"/>
       <c r="D146" s="83" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E146" s="40"/>
       <c r="F146" s="40"/>
@@ -6503,7 +6487,7 @@
       <c r="B147" s="17"/>
       <c r="C147" s="145"/>
       <c r="D147" s="83" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E147" s="40"/>
       <c r="F147" s="41"/>
@@ -6516,11 +6500,11 @@
       </c>
       <c r="C148" s="146"/>
       <c r="D148" s="147" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E148" s="40"/>
       <c r="F148" s="148" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G148" s="38"/>
     </row>
@@ -6531,7 +6515,7 @@
       </c>
       <c r="C149" s="17"/>
       <c r="D149" s="30" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E149" s="40"/>
       <c r="F149" s="41"/>
@@ -6544,7 +6528,7 @@
       <c r="C150" s="17"/>
       <c r="D150" s="40"/>
       <c r="E150" s="40"/>
-      <c r="F150" s="114"/>
+      <c r="F150" s="115"/>
     </row>
     <row r="151" ht="18.75" customHeight="1">
       <c r="A151" s="21"/>
@@ -6560,13 +6544,13 @@
       </c>
       <c r="C152" s="17"/>
       <c r="D152" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="E152" s="30" t="s">
         <v>202</v>
       </c>
-      <c r="E152" s="30" t="s">
+      <c r="G152" s="46" t="s">
         <v>203</v>
-      </c>
-      <c r="G152" s="46" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="153" ht="93.75" customHeight="1">
@@ -6584,15 +6568,15 @@
       </c>
       <c r="C154" s="17"/>
       <c r="D154" s="58" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E154" s="40"/>
       <c r="F154" s="64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G154" s="41"/>
       <c r="H154" s="56" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="155" ht="34.5" customHeight="1">
@@ -6601,8 +6585,8 @@
       <c r="C155" s="17"/>
       <c r="D155" s="41"/>
       <c r="E155" s="40"/>
-      <c r="F155" s="124" t="s">
-        <v>207</v>
+      <c r="F155" s="125" t="s">
+        <v>206</v>
       </c>
       <c r="G155" s="38"/>
       <c r="H155" s="40"/>
@@ -6613,13 +6597,13 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="C156" s="17"/>
-      <c r="D156" s="124" t="s">
-        <v>208</v>
+      <c r="D156" s="125" t="s">
+        <v>207</v>
       </c>
       <c r="E156" s="40"/>
       <c r="F156" s="40"/>
-      <c r="G156" s="117" t="s">
-        <v>209</v>
+      <c r="G156" s="118" t="s">
+        <v>208</v>
       </c>
       <c r="H156" s="40"/>
     </row>
@@ -6630,7 +6614,7 @@
       <c r="D157" s="41"/>
       <c r="E157" s="41"/>
       <c r="F157" s="150" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G157" s="40"/>
       <c r="H157" s="40"/>
@@ -6642,14 +6626,14 @@
       </c>
       <c r="C158" s="17"/>
       <c r="D158" s="151" t="s">
+        <v>210</v>
+      </c>
+      <c r="E158" s="56" t="s">
         <v>211</v>
-      </c>
-      <c r="E158" s="56" t="s">
-        <v>212</v>
       </c>
       <c r="F158" s="39"/>
       <c r="G158" s="152" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H158" s="40"/>
     </row>
@@ -6658,7 +6642,7 @@
       <c r="B159" s="40"/>
       <c r="C159" s="17"/>
       <c r="D159" s="58" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E159" s="40"/>
       <c r="G159" s="40"/>
@@ -6714,13 +6698,9 @@
       <c r="D164" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="329">
+  <mergeCells count="328">
     <mergeCell ref="B118:B119"/>
     <mergeCell ref="B120:B121"/>
-    <mergeCell ref="C131:C141"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="D138:D141"/>
     <mergeCell ref="B107:B108"/>
     <mergeCell ref="B109:B110"/>
     <mergeCell ref="C109:C112"/>
@@ -6728,6 +6708,32 @@
     <mergeCell ref="C113:C121"/>
     <mergeCell ref="B114:B115"/>
     <mergeCell ref="B116:B117"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="D149:D151"/>
+    <mergeCell ref="D152:D153"/>
+    <mergeCell ref="D154:D155"/>
+    <mergeCell ref="D156:D157"/>
+    <mergeCell ref="D159:D160"/>
+    <mergeCell ref="D161:D164"/>
+    <mergeCell ref="C131:C141"/>
+    <mergeCell ref="C142:C144"/>
+    <mergeCell ref="C145:C146"/>
+    <mergeCell ref="C148:C164"/>
+    <mergeCell ref="B131:B132"/>
+    <mergeCell ref="B146:B147"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="B154:B155"/>
+    <mergeCell ref="B156:B157"/>
+    <mergeCell ref="B158:B159"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="D126:D127"/>
+    <mergeCell ref="B128:B129"/>
+    <mergeCell ref="D128:D129"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D142:D143"/>
     <mergeCell ref="D51:D52"/>
     <mergeCell ref="D53:D54"/>
     <mergeCell ref="D45:D46"/>
@@ -6759,98 +6765,139 @@
     <mergeCell ref="D114:D115"/>
     <mergeCell ref="D116:D117"/>
     <mergeCell ref="D118:D119"/>
+    <mergeCell ref="D91:D94"/>
+    <mergeCell ref="D95:D101"/>
     <mergeCell ref="D77:D78"/>
     <mergeCell ref="D79:D82"/>
-    <mergeCell ref="D83:D84"/>
     <mergeCell ref="C89:D89"/>
     <mergeCell ref="C90:C107"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="D92:D101"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="B131:B132"/>
+    <mergeCell ref="D87:D88"/>
+    <mergeCell ref="D85:D86"/>
+    <mergeCell ref="L94:L104"/>
+    <mergeCell ref="L105:L117"/>
+    <mergeCell ref="J101:J110"/>
+    <mergeCell ref="J111:J115"/>
+    <mergeCell ref="I105:I112"/>
+    <mergeCell ref="I113:I115"/>
+    <mergeCell ref="M111:M114"/>
+    <mergeCell ref="M115:M117"/>
+    <mergeCell ref="I90:I93"/>
+    <mergeCell ref="I94:I104"/>
+    <mergeCell ref="J94:J100"/>
+    <mergeCell ref="K94:K106"/>
+    <mergeCell ref="M96:M110"/>
+    <mergeCell ref="K107:K113"/>
+    <mergeCell ref="K114:K117"/>
+    <mergeCell ref="J116:J117"/>
+    <mergeCell ref="O101:O125"/>
+    <mergeCell ref="O126:O129"/>
+    <mergeCell ref="M131:M164"/>
+    <mergeCell ref="N131:N138"/>
+    <mergeCell ref="O131:O133"/>
+    <mergeCell ref="O134:O164"/>
+    <mergeCell ref="N139:N164"/>
+    <mergeCell ref="P139:P164"/>
+    <mergeCell ref="N96:N115"/>
+    <mergeCell ref="P101:P117"/>
+    <mergeCell ref="N116:N119"/>
+    <mergeCell ref="P118:P129"/>
+    <mergeCell ref="N120:N121"/>
+    <mergeCell ref="N122:N123"/>
+    <mergeCell ref="N124:N129"/>
+    <mergeCell ref="P131:P138"/>
+    <mergeCell ref="J126:J129"/>
+    <mergeCell ref="I130:K130"/>
+    <mergeCell ref="E126:E127"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="G126:G127"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="I126:I127"/>
+    <mergeCell ref="E128:E129"/>
+    <mergeCell ref="G128:G129"/>
+    <mergeCell ref="J81:J84"/>
+    <mergeCell ref="J85:J88"/>
+    <mergeCell ref="J90:J93"/>
+    <mergeCell ref="K90:K93"/>
+    <mergeCell ref="L90:L93"/>
+    <mergeCell ref="M90:M94"/>
+    <mergeCell ref="N90:N94"/>
+    <mergeCell ref="O90:O93"/>
+    <mergeCell ref="G79:G82"/>
+    <mergeCell ref="H79:H82"/>
+    <mergeCell ref="I81:I82"/>
+    <mergeCell ref="G83:G88"/>
+    <mergeCell ref="H83:H84"/>
+    <mergeCell ref="I84:I88"/>
+    <mergeCell ref="H85:H88"/>
+    <mergeCell ref="K118:K121"/>
+    <mergeCell ref="K122:K125"/>
+    <mergeCell ref="L122:L125"/>
+    <mergeCell ref="M124:M127"/>
+    <mergeCell ref="K126:K127"/>
+    <mergeCell ref="L126:L129"/>
+    <mergeCell ref="K128:K129"/>
+    <mergeCell ref="M128:M129"/>
+    <mergeCell ref="F122:F123"/>
+    <mergeCell ref="F124:F125"/>
+    <mergeCell ref="I124:I125"/>
+    <mergeCell ref="J124:J125"/>
+    <mergeCell ref="F94:F102"/>
+    <mergeCell ref="F103:F104"/>
+    <mergeCell ref="F105:F106"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="F107:F113"/>
+    <mergeCell ref="E109:E113"/>
+    <mergeCell ref="F114:F121"/>
+    <mergeCell ref="E96:E102"/>
     <mergeCell ref="E131:E132"/>
-    <mergeCell ref="F131:F133"/>
-    <mergeCell ref="G131:G134"/>
     <mergeCell ref="E133:E134"/>
-    <mergeCell ref="D126:D127"/>
-    <mergeCell ref="D128:D129"/>
     <mergeCell ref="F134:F141"/>
     <mergeCell ref="E135:E136"/>
     <mergeCell ref="E137:E138"/>
     <mergeCell ref="E139:E140"/>
     <mergeCell ref="E141:E144"/>
-    <mergeCell ref="E114:E116"/>
-    <mergeCell ref="E118:E119"/>
-    <mergeCell ref="D120:D123"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="C122:C124"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="F122:F123"/>
-    <mergeCell ref="K126:K127"/>
-    <mergeCell ref="K128:K129"/>
-    <mergeCell ref="K131:K132"/>
-    <mergeCell ref="K133:K136"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="G126:G127"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="I126:I127"/>
-    <mergeCell ref="J126:J129"/>
-    <mergeCell ref="L126:L129"/>
-    <mergeCell ref="G128:G129"/>
-    <mergeCell ref="I130:K130"/>
-    <mergeCell ref="D124:D125"/>
-    <mergeCell ref="E124:E125"/>
-    <mergeCell ref="F124:F125"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="E126:E127"/>
-    <mergeCell ref="B128:B129"/>
-    <mergeCell ref="E128:E129"/>
+    <mergeCell ref="F81:F84"/>
+    <mergeCell ref="F85:F88"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="E83:E87"/>
+    <mergeCell ref="H90:H102"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="F131:F133"/>
+    <mergeCell ref="G131:G134"/>
     <mergeCell ref="I131:I134"/>
     <mergeCell ref="J131:J133"/>
+    <mergeCell ref="K131:K132"/>
     <mergeCell ref="L131:L133"/>
+    <mergeCell ref="K133:K136"/>
+    <mergeCell ref="G135:G139"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="G162:G164"/>
     <mergeCell ref="H131:H133"/>
     <mergeCell ref="H134:H136"/>
-    <mergeCell ref="G135:G139"/>
-    <mergeCell ref="C142:C144"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="F158:F164"/>
-    <mergeCell ref="D159:D160"/>
-    <mergeCell ref="D161:D164"/>
-    <mergeCell ref="E162:E164"/>
-    <mergeCell ref="G162:G164"/>
+    <mergeCell ref="L134:L164"/>
+    <mergeCell ref="K137:K164"/>
+    <mergeCell ref="F144:F147"/>
+    <mergeCell ref="F148:F149"/>
+    <mergeCell ref="F150:F153"/>
     <mergeCell ref="H162:H164"/>
     <mergeCell ref="I135:I140"/>
     <mergeCell ref="I141:I143"/>
-    <mergeCell ref="F144:F147"/>
-    <mergeCell ref="C145:C146"/>
-    <mergeCell ref="C148:C164"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="F155:F156"/>
-    <mergeCell ref="H103:H104"/>
-    <mergeCell ref="H105:H108"/>
-    <mergeCell ref="I105:I112"/>
-    <mergeCell ref="H109:H110"/>
-    <mergeCell ref="H111:H112"/>
-    <mergeCell ref="I113:I115"/>
-    <mergeCell ref="I116:I119"/>
+    <mergeCell ref="J134:J164"/>
+    <mergeCell ref="I144:I164"/>
     <mergeCell ref="H137:H144"/>
     <mergeCell ref="H145:H153"/>
-    <mergeCell ref="F148:F149"/>
+    <mergeCell ref="G140:G147"/>
     <mergeCell ref="G148:G151"/>
-    <mergeCell ref="B146:B147"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="B152:B153"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="B156:B157"/>
-    <mergeCell ref="B158:B159"/>
-    <mergeCell ref="D149:D151"/>
-    <mergeCell ref="D152:D153"/>
+    <mergeCell ref="E145:E151"/>
     <mergeCell ref="E152:E157"/>
-    <mergeCell ref="D154:D155"/>
-    <mergeCell ref="D156:D157"/>
-    <mergeCell ref="E145:E151"/>
     <mergeCell ref="E158:E161"/>
+    <mergeCell ref="E162:E164"/>
+    <mergeCell ref="G152:G154"/>
+    <mergeCell ref="H154:H161"/>
+    <mergeCell ref="G156:G157"/>
+    <mergeCell ref="F155:F156"/>
+    <mergeCell ref="F158:F164"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="D11:D14"/>
     <mergeCell ref="E11:E14"/>
@@ -6896,12 +6943,30 @@
     <mergeCell ref="G64:G65"/>
     <mergeCell ref="G66:G70"/>
     <mergeCell ref="I74:I76"/>
+    <mergeCell ref="O60:O76"/>
+    <mergeCell ref="O77:O80"/>
+    <mergeCell ref="M60:M78"/>
+    <mergeCell ref="M79:M82"/>
+    <mergeCell ref="N75:N86"/>
+    <mergeCell ref="O81:O84"/>
+    <mergeCell ref="P90:P100"/>
+    <mergeCell ref="O94:O100"/>
+    <mergeCell ref="L78:L84"/>
+    <mergeCell ref="L85:L88"/>
+    <mergeCell ref="M83:M86"/>
+    <mergeCell ref="M87:M88"/>
+    <mergeCell ref="L60:L76"/>
+    <mergeCell ref="N60:N68"/>
+    <mergeCell ref="P60:P75"/>
+    <mergeCell ref="N69:N74"/>
+    <mergeCell ref="P76:P88"/>
+    <mergeCell ref="K81:K88"/>
+    <mergeCell ref="O85:O88"/>
+    <mergeCell ref="N87:N88"/>
     <mergeCell ref="E49:E54"/>
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="E60:E61"/>
     <mergeCell ref="E73:E79"/>
-    <mergeCell ref="E80:E83"/>
-    <mergeCell ref="E84:E88"/>
     <mergeCell ref="D26:D29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D31:D34"/>
@@ -6918,7 +6983,6 @@
     <mergeCell ref="C85:C88"/>
     <mergeCell ref="D56:D58"/>
     <mergeCell ref="D69:D72"/>
-    <mergeCell ref="D85:D88"/>
     <mergeCell ref="K60:K75"/>
     <mergeCell ref="K76:K79"/>
     <mergeCell ref="I77:I80"/>
@@ -6930,120 +6994,39 @@
     <mergeCell ref="H75:H78"/>
     <mergeCell ref="F76:F78"/>
     <mergeCell ref="F79:F80"/>
-    <mergeCell ref="N96:N115"/>
-    <mergeCell ref="M111:M114"/>
-    <mergeCell ref="P101:P117"/>
-    <mergeCell ref="P118:P129"/>
-    <mergeCell ref="P131:P138"/>
-    <mergeCell ref="P139:P164"/>
-    <mergeCell ref="O85:O88"/>
-    <mergeCell ref="M87:M88"/>
-    <mergeCell ref="N87:N88"/>
-    <mergeCell ref="P90:P100"/>
-    <mergeCell ref="O94:O100"/>
-    <mergeCell ref="O101:O125"/>
-    <mergeCell ref="N120:N121"/>
-    <mergeCell ref="N122:N123"/>
-    <mergeCell ref="O126:O129"/>
-    <mergeCell ref="O131:O133"/>
-    <mergeCell ref="O134:O164"/>
-    <mergeCell ref="N131:N138"/>
-    <mergeCell ref="N139:N164"/>
-    <mergeCell ref="M118:M121"/>
-    <mergeCell ref="M122:M123"/>
-    <mergeCell ref="M124:M127"/>
-    <mergeCell ref="M128:M129"/>
-    <mergeCell ref="N124:N129"/>
-    <mergeCell ref="M131:M164"/>
-    <mergeCell ref="J81:J84"/>
-    <mergeCell ref="J85:J88"/>
-    <mergeCell ref="J90:J93"/>
-    <mergeCell ref="L90:L93"/>
-    <mergeCell ref="M90:M94"/>
-    <mergeCell ref="N90:N94"/>
-    <mergeCell ref="O90:O93"/>
-    <mergeCell ref="G79:G82"/>
-    <mergeCell ref="H79:H82"/>
-    <mergeCell ref="I81:I82"/>
-    <mergeCell ref="G83:G88"/>
-    <mergeCell ref="H83:H84"/>
-    <mergeCell ref="I84:I88"/>
-    <mergeCell ref="H85:H88"/>
     <mergeCell ref="G90:G93"/>
     <mergeCell ref="G94:G104"/>
     <mergeCell ref="G105:G108"/>
     <mergeCell ref="G110:G111"/>
     <mergeCell ref="G113:G115"/>
     <mergeCell ref="G116:G119"/>
+    <mergeCell ref="H103:H104"/>
+    <mergeCell ref="H105:H108"/>
+    <mergeCell ref="H109:H110"/>
+    <mergeCell ref="H111:H112"/>
+    <mergeCell ref="H113:H116"/>
+    <mergeCell ref="I116:I119"/>
+    <mergeCell ref="H118:H119"/>
+    <mergeCell ref="I120:I121"/>
+    <mergeCell ref="I122:I123"/>
     <mergeCell ref="G120:G122"/>
     <mergeCell ref="G123:G124"/>
-    <mergeCell ref="I90:I93"/>
-    <mergeCell ref="I94:I104"/>
-    <mergeCell ref="J94:J100"/>
     <mergeCell ref="J118:J121"/>
-    <mergeCell ref="K118:K121"/>
     <mergeCell ref="L118:L121"/>
-    <mergeCell ref="I120:I121"/>
-    <mergeCell ref="F81:F84"/>
-    <mergeCell ref="F85:F88"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="E91:E94"/>
-    <mergeCell ref="H94:H102"/>
-    <mergeCell ref="E95:E102"/>
-    <mergeCell ref="F94:F102"/>
-    <mergeCell ref="F103:F104"/>
-    <mergeCell ref="F105:F106"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="F107:F113"/>
-    <mergeCell ref="E109:E113"/>
-    <mergeCell ref="F114:F121"/>
+    <mergeCell ref="M118:M121"/>
     <mergeCell ref="H120:H121"/>
     <mergeCell ref="H122:H124"/>
-    <mergeCell ref="I122:I123"/>
     <mergeCell ref="J122:J123"/>
-    <mergeCell ref="K122:K125"/>
-    <mergeCell ref="L122:L125"/>
-    <mergeCell ref="I124:I125"/>
-    <mergeCell ref="J124:J125"/>
-    <mergeCell ref="G152:G154"/>
-    <mergeCell ref="H154:H161"/>
-    <mergeCell ref="G156:G157"/>
-    <mergeCell ref="G158:G161"/>
-    <mergeCell ref="H113:H116"/>
-    <mergeCell ref="H118:H119"/>
-    <mergeCell ref="J134:J164"/>
-    <mergeCell ref="L134:L164"/>
-    <mergeCell ref="K137:K164"/>
-    <mergeCell ref="G140:G147"/>
-    <mergeCell ref="I144:I164"/>
-    <mergeCell ref="K90:K93"/>
-    <mergeCell ref="K94:K106"/>
-    <mergeCell ref="K81:K88"/>
-    <mergeCell ref="L85:L88"/>
-    <mergeCell ref="L94:L104"/>
-    <mergeCell ref="J101:J110"/>
-    <mergeCell ref="L105:L117"/>
-    <mergeCell ref="J111:J115"/>
-    <mergeCell ref="J116:J117"/>
-    <mergeCell ref="M60:M78"/>
-    <mergeCell ref="M79:M82"/>
-    <mergeCell ref="M96:M110"/>
-    <mergeCell ref="L78:L84"/>
-    <mergeCell ref="M83:M86"/>
-    <mergeCell ref="K107:K113"/>
-    <mergeCell ref="K114:K117"/>
-    <mergeCell ref="M115:M117"/>
-    <mergeCell ref="N116:N119"/>
-    <mergeCell ref="O60:O76"/>
-    <mergeCell ref="L60:L76"/>
-    <mergeCell ref="N60:N68"/>
-    <mergeCell ref="P60:P75"/>
-    <mergeCell ref="N69:N74"/>
-    <mergeCell ref="N75:N86"/>
-    <mergeCell ref="P76:P88"/>
-    <mergeCell ref="O81:O84"/>
-    <mergeCell ref="O77:O80"/>
+    <mergeCell ref="M122:M123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="E114:E116"/>
+    <mergeCell ref="E118:E119"/>
+    <mergeCell ref="D120:D123"/>
+    <mergeCell ref="C122:C124"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="D124:D125"/>
+    <mergeCell ref="E124:E125"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId4" ref="F148"/>
@@ -7072,21 +7055,21 @@
   <sheetData>
     <row r="1">
       <c r="B1" s="153" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="153" t="s">
         <v>215</v>
       </c>
-      <c r="C1" s="153" t="s">
+      <c r="D1" s="153" t="s">
         <v>216</v>
       </c>
-      <c r="D1" s="153" t="s">
+      <c r="E1" s="153" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="153" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="154" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B2" s="155"/>
       <c r="C2" s="155"/>
@@ -7118,32 +7101,32 @@
     <row r="3">
       <c r="A3" s="157"/>
       <c r="B3" s="153" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" s="153" t="s">
         <v>220</v>
-      </c>
-      <c r="E3" s="153" t="s">
-        <v>221</v>
       </c>
       <c r="AA3" s="158"/>
     </row>
     <row r="4">
       <c r="A4" s="157"/>
       <c r="B4" s="153" t="s">
+        <v>221</v>
+      </c>
+      <c r="E4" s="153" t="s">
         <v>222</v>
-      </c>
-      <c r="E4" s="153" t="s">
-        <v>223</v>
       </c>
       <c r="AA4" s="158"/>
     </row>
     <row r="5">
       <c r="A5" s="159"/>
       <c r="B5" s="160" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C5" s="161"/>
       <c r="D5" s="161"/>
       <c r="E5" s="160" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F5" s="161"/>
       <c r="G5" s="161"/>
@@ -7170,7 +7153,7 @@
     </row>
     <row r="6">
       <c r="A6" s="154" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B6" s="163"/>
       <c r="C6" s="155"/>
@@ -7202,51 +7185,51 @@
     <row r="7">
       <c r="A7" s="157"/>
       <c r="B7" s="153" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" s="153" t="s">
         <v>227</v>
-      </c>
-      <c r="E7" s="153" t="s">
-        <v>228</v>
       </c>
       <c r="AA7" s="158"/>
     </row>
     <row r="8">
       <c r="A8" s="157"/>
       <c r="B8" s="153" t="s">
+        <v>228</v>
+      </c>
+      <c r="E8" s="153" t="s">
         <v>229</v>
-      </c>
-      <c r="E8" s="153" t="s">
-        <v>230</v>
       </c>
       <c r="AA8" s="158"/>
     </row>
     <row r="9">
       <c r="A9" s="157"/>
       <c r="B9" s="153" t="s">
+        <v>230</v>
+      </c>
+      <c r="E9" s="153" t="s">
         <v>231</v>
-      </c>
-      <c r="E9" s="153" t="s">
-        <v>232</v>
       </c>
       <c r="AA9" s="158"/>
     </row>
     <row r="10">
       <c r="A10" s="157"/>
       <c r="B10" s="153" t="s">
+        <v>232</v>
+      </c>
+      <c r="E10" s="153" t="s">
         <v>233</v>
-      </c>
-      <c r="E10" s="153" t="s">
-        <v>234</v>
       </c>
       <c r="AA10" s="158"/>
     </row>
     <row r="11">
       <c r="A11" s="159"/>
       <c r="B11" s="160" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D11" s="161"/>
       <c r="E11" s="160" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F11" s="161"/>
       <c r="G11" s="161"/>
@@ -7273,7 +7256,7 @@
     </row>
     <row r="12">
       <c r="A12" s="154" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B12" s="155"/>
       <c r="C12" s="155"/>
@@ -7305,22 +7288,22 @@
     <row r="13">
       <c r="A13" s="157"/>
       <c r="B13" s="153" t="s">
+        <v>237</v>
+      </c>
+      <c r="E13" s="153" t="s">
         <v>238</v>
-      </c>
-      <c r="E13" s="153" t="s">
-        <v>239</v>
       </c>
       <c r="AA13" s="158"/>
     </row>
     <row r="14">
       <c r="A14" s="159"/>
       <c r="B14" s="160" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C14" s="161"/>
       <c r="D14" s="161"/>
       <c r="E14" s="160" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F14" s="161"/>
       <c r="G14" s="161"/>
@@ -7347,7 +7330,7 @@
     </row>
     <row r="15">
       <c r="A15" s="154" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B15" s="155"/>
       <c r="C15" s="155"/>
@@ -7378,10 +7361,10 @@
     </row>
     <row r="16">
       <c r="A16" s="164" t="s">
+        <v>242</v>
+      </c>
+      <c r="B16" s="153" t="s">
         <v>243</v>
-      </c>
-      <c r="B16" s="153" t="s">
-        <v>244</v>
       </c>
       <c r="AA16" s="158"/>
     </row>
@@ -7390,25 +7373,25 @@
         <v>6</v>
       </c>
       <c r="B17" s="153" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="AA17" s="158"/>
     </row>
     <row r="18">
       <c r="A18" s="164" t="s">
+        <v>245</v>
+      </c>
+      <c r="B18" s="153" t="s">
         <v>246</v>
-      </c>
-      <c r="B18" s="153" t="s">
-        <v>247</v>
       </c>
       <c r="AA18" s="158"/>
     </row>
     <row r="19">
       <c r="A19" s="165" t="s">
+        <v>247</v>
+      </c>
+      <c r="B19" s="160" t="s">
         <v>248</v>
-      </c>
-      <c r="B19" s="160" t="s">
-        <v>249</v>
       </c>
       <c r="C19" s="161"/>
       <c r="D19" s="161"/>
@@ -7438,27 +7421,27 @@
     </row>
     <row r="20">
       <c r="A20" s="153" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="153" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="166" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="166" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="166" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ingested and formatted new schedule, mapping to locations. Source of truth for Schedule is now the_real_schedule_events.json
</commit_message>
<xml_diff>
--- a/THE (REAL) SCHEDULE.xlsx
+++ b/THE (REAL) SCHEDULE.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={dbc866ff-36c2-4b34-a443-fd7ab61a53ab}</author>
+    <author>tc={1a9a9bfc-57a7-4d31-a9a1-1f06d07d8acf}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{dbc866ff-36c2-4b34-a443-fd7ab61a53ab}" ref="D53">
+    <comment authorId="0" xr:uid="{1a9a9bfc-57a7-4d31-a9a1-1f06d07d8acf}" ref="D53">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="258">
   <si>
     <t>LAST UPDATED 3/24/26 3 PM PST</t>
   </si>
@@ -161,7 +161,8 @@
     <t>Little Little Italy Italian Festival
 Apertivo &amp; Film Screening
 6-7:30 PM
-Little Little Italy</t>
+Little Little Italy
+Have an old school italian festival with music food and drink (aperitivo) during sunset and then screen from Rome Italy, Anna Negri's, Venice Film Festival selected, feature Documentary. Toni mio Padre afterwards with Q&amp;A</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -235,36 +236,15 @@
     <t>3D Therapy in Perspective
 5-7 PM
 3D
-Gallery Opening by Jimmy Mahafee</t>
+Gallery Opening by Jimmy Mahafee
+“built of art like legos on 4'x6' panels, the installation is composed of 250 paintings digitized onto coreplast. this habitrail of my imagination is a construction of the places people and art i love so much I had to paint a picture of them and build them a cappella.“</t>
   </si>
   <si>
     <t>The Magic Carpet Ride
 6-10 PM
 TBD
-AV Experience</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">The Nest Opening Ceremony
-by Debra Berger &amp; Erica Spooner
-7-8 PM
-The Nest
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>Celebrating a fiber sculpture of soft emergence.</t>
-    </r>
+AV Experience
+“A 6-minute blindfolded journey on a magic carpet. EEG captures how your nervous system responds to surrender, rhythm, mystery, being seen — and translates it into four glyphs sealed in wax. Your frequency fingerprint. The quest: find the others on your wavelength.”</t>
   </si>
   <si>
     <r>
@@ -302,7 +282,8 @@
     <t>Butterfly Pavilion
 8-9 PM
 Butterfly Pavillion
-Gallery Opening by April Leighton</t>
+Gallery Opening by April Leighton
+“The Butterfly Pavilion is an immersive experience created with colorful origami butterflies and flowers and lights creating a fantasy experience”</t>
   </si>
   <si>
     <r>
@@ -344,7 +325,8 @@
     <t>Artemis makes a housecall 
 9-10 PM
 Gallery Opening by Branwen
-The Institute</t>
+The Institute
+“In my surrealist conceptual offering I'm bringing magic and symbolism to the Salton Sea by inviting Artemis, the lady of the lake, to visit her home away from home, a hollow Redwood tree temple in a trailer, thus shifting shapes and playing with perception.”</t>
   </si>
   <si>
     <t>"Last Flight Home" 
@@ -378,7 +360,9 @@
     <t>The Salton Sea Museum &amp; Library
 8 AM-2 PM
 BBAC
-Curated by Christopher Landis</t>
+Curated by Christopher Landis
+“Reopening at BBAC the Salton Sea Museum and Library has added new ephemera and titles representing the Salton Sea history and ecology. 
+Additionally titles include topics covering Western Water, Deserts and Landscape studies."</t>
   </si>
   <si>
     <t xml:space="preserve">Mapping the Sacrifice Zone: 
@@ -548,26 +532,10 @@
 Museum of Unwanted Architecture</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">The Silvertongued Devil Speaks
+    <t>The Silvertongued Devil Speaks
 4-5pm
 Horsefly Ranch
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>A talking robot made from discarded music equipment offers free flattery for artists, lovers, and tyrants. Choose your poison.</t>
-    </r>
+“The Silver Tongued Devil: A Speaker-Creature is an interactive sound sculpture constructed out of broken music equipment collected by a recently-deceased San Diego musician. Visit the Creature to hear angels plummeting into the Underworld—and to receive your own flattering fortune!”</t>
   </si>
   <si>
     <r>
@@ -692,7 +660,8 @@
     <t>Birth, Life and Becoming
 by Cactus Chaos &amp; Kamau
 6-8 PM
-Jaybird Nest</t>
+Jaybird Nest
+“The Thread of Life | Act III: Own Your Fate” is an immersive ritual-performance where myth, ancestry, and craft colide. Guided by Nyx and the Moirai, participants are invited to own their fate and weave it into the Loom of Life.”</t>
   </si>
   <si>
     <r>
@@ -750,29 +719,14 @@
 AV Experience</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">The Last Party 
+    <t>The Last Party 
 Gallery Opening
 7 PM-11 PM
 Open Gallery Hours
 FOUNDATION FOUNDATION
 Curated by Greg Haberny
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>feat. Adam Cullins, Jack Parker, Randy Polumbo, Judith Berndsen, Sean Guerrero, Masha D’yans, Jake Wade, Bunny Valentine, Bill Saylor, Camille Schefter, Nick Fari, Steve Hash, Brett Lindell, Katrina Brown, Bob Swanek, Joe Regan, Tafka J. Lighthouse, Stephanie Caite, Greg Haberny, Heidl Hasenauer</t>
-    </r>
+feat. Adam Cullins, Jack Parker, Randy Polumbo, Judith Berndsen, Sean Guerrero, Masha D’yans, Jake Wade, Bunny Valentine, Bill Saylor, Camille Schefter, Nick Fari, Steve Hash, Brett Lindell, Katrina Brown, Bob Swanek, Joe Regan, Tafka J. Lighthouse, Stephanie Caite, Greg Haberny, Heidl Hasenauer\
+“We will be making a show diverse in personalities and disciplines. The setting will be a smorgasbord of delights for the senses.”</t>
   </si>
   <si>
     <t>Sunset DJ &amp; Cocktail Hour
@@ -841,13 +795,15 @@
 Drag Show
 + Care Club
 7:30-9:30 PM
-Temple to the Scientific Method</t>
+Temple to the Scientific Method
+“Glorious Holy Kings is a drag show highlighting Kings uniquely designed for Bombay Beach. The Queer community has faced many judgements through the years, and not one of them has stopped us from celebrating our most authentic selves! Kingdom comes in the land of milk, honey, and drag. “</t>
   </si>
   <si>
     <t>The Social Equilibrium Calibration Unit
 by Damon James Duke
 7-7:30 PM
-The Beach</t>
+The Beach
+“Time is running.”</t>
   </si>
   <si>
     <r>
@@ -891,20 +847,16 @@
 BBIFF</t>
   </si>
   <si>
-    <t xml:space="preserve">S.S.S.S.S's Shared Telescope Sesh
+    <t>S.S.S.S.S's Shared Telescope Sesh
 by Salton Sea Stellar Sky Society
 8-9 PM
-Start Sight Site, Bombay North </t>
+Start Sight Site, Bombay North 
+“The Salton Sea Stellar Sky Society’s Star Sight Site: a shared sculptural sanctuary supplying stargazing, star-seeking, skyward study, and speculative celestial storytelling for the Bombay Beach community. Styled and supported by The 9-foot Comeback Cube by Gregg Fleishman.”</t>
   </si>
   <si>
     <t>Care Club
 10 PM-2 AM
 Club 86</t>
-  </si>
-  <si>
-    <t>Karaoke
-8 PM-1 AM
-The Ski Inn</t>
   </si>
   <si>
     <r>
@@ -1008,37 +960,13 @@
 The Tradewinds</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>Algo(g)rave: The Manual for Dying
+    <t>Algo(g)rave: The Manual for Dying
 by Katana Calderwood
 Alejandro Sanchez-Medina: Audio Engineer
- Martians: Audio Artists</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">10 PM-12 AM
+ Martians: Audio Artists
+10 PM-12 AM
 RaphaLots
-</t>
-    </r>
+“Death is inevitable, but the true horror is the infinite return. Inspired by Buddhist earthly hells, Algo(g)rave explores possibilities of disrupting the material-time mesh network of life. To escape the cycle, we move through recursive loops toward white noise—the soul’s final, static resolution.”</t>
   </si>
   <si>
     <t>The Last Canter
@@ -1156,7 +1084,8 @@
     <t>Mella Tarantella--Risorga e Balla 
 con i Morti e Vivi alla Fine Dei Giorni
 12-2 AM
-PoP</t>
+PoP 
+"Dance for the End of Days"</t>
   </si>
   <si>
     <r>
@@ -1187,26 +1116,17 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">The Jazz Club*
+    <t>The Jazz Club*
 12:30-2:30 AM
 sponsored by Yarger Projects feat. Tyler Hammond Jazz Experience
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>the DoRD, Estates</t>
-    </r>
+the DoRD, Estates
+“The Jazz Club at the DORD has added another remarkable musical experience to BBB , paralleling the The Opera, The Ballet  at the DJ sets …”</t>
+  </si>
+  <si>
+    <t>The Salton Sea Museum &amp; Library
+8 AM-2 PM
+BBAC
+Curated by Christopher Landis</t>
   </si>
   <si>
     <r>
@@ -1291,7 +1211,8 @@
     <t>okay you*
 10-11 AM
 Henderson Hall 
-Morning Movement Practice with Clifford</t>
+Morning Movement Practice with Clifford
+"okay you, you're ok. Come breathe, stretch, and start your day with one of the oldest calm technologies: gentle yoga and ambient music designed to develop interoceptive awareness and genuine presence. No experience necessary. Bring a mat if you have one."</t>
   </si>
   <si>
     <r>
@@ -1317,35 +1238,28 @@
     <t>AI &amp; The Apocalyptic Imagination
 11 AM-12 PM
 No Shoes, Institute
-Lecture by rina nicolae</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Quesadilla Communion
+Lecture by rina nicolae
+“AI is our era's apocalyptic narrative. This talk traces how the eschatological frame operates as both a belief system and a power structure, concentrating authority in those who claim to understand the coming transformation. how can we engage with the change without submitting to this mythology?”</t>
+  </si>
+  <si>
+    <t>Quesadilla Communion
 by Isaac Taylor
 11 AM-12 PM
 Temple to the Scientific Method
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>Queso, Kool-Aid, and Comedy with Rev. Earl E. Gaytes</t>
-    </r>
+Queso, Kool-Aid, and Comedy with Rev. Earl E. Gaytes
+“Come to Cheesus” in an Old Time Religion styled tent revival as Rev. Earl E. Gaytes preaches about the one true whey of salvation. Expect a cheesy sermon, boxed wine communion, some food &amp; fellowship to follow.”</t>
   </si>
   <si>
     <t>Care Club
 11 AM-1 PM
 Temple to the Scientific Method</t>
+  </si>
+  <si>
+    <t>Vibroacoustic Experience*
+11 AM-1 PM
+Westlandia Desert Oasis
+(The Beach)
+“Tired of wandering through life? Pause and arrive at Westlandia Desert Oasis, where weary feet and restless minds find renewal. Heal in our vibroacoustic dome, sip a last-call drink in the lounge, and leave your mark by gifting found objects to our vibrant peddlers’ paradise.”</t>
   </si>
   <si>
     <t>Burger Burn Fundraiser
@@ -1382,45 +1296,23 @@
     <t>God / Is
 Performance by Courtney Alexander
 11:30 AM-12:30 PM
-Dream Demon</t>
+Dream Demon
+“God Is / Sustenance centers the body and land as sacred sites. A living altar invites offering and reflection on embodied divinity, while immersive stations throughout the landscape guide participants into contemplation, reverence, and renewed relationship with the environment.”</t>
   </si>
   <si>
     <t>An information-theoretic recapitulation of God in the form of a public figure
 Lecture by Leo Christov-Moore
 12-1 PM
 No Shoes, Institute
-Philosophy Conference</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">Sunshine Dreams:
+Philosophy Conference
+“a public figure : from the conditions of embodiment -vulnerability, mortality, open, endedness, we get intrinsic Drives to maximize complexity on multiple scales, advocating for an epistemic/homeostatic value in cultivating trust on infinite spacetimehorizons, towards the empowerment of all things.”</t>
+  </si>
+  <si>
+    <t>Sunshine Dreams:
 Legends of Bombay Beach, Unconditional Love and Stuff
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">12-5 PM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Henderson Hall</t>
-    </r>
+12-5 PM
+Henderson Hall
+"An excursion through the essence of Bombay Beach led by the souls of those that lived it.”</t>
   </si>
   <si>
     <r>
@@ -1484,41 +1376,29 @@
 1-2 PM
 The Portal, The Institute
 Marc Vinciguerra
-Philosophy Conference</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Derangers Before the Playa
+Philosophy Conference
+“The Philosophical Computer is a philosophical sculpture entirely permutable that is made of 54 symbols of the great philosophical revolutions of the western world from the totemic God to Post-modernity. The goal is to articulate these symbols together to create new contemporary cultural synthesis.”</t>
+  </si>
+  <si>
+    <t>Derangers Before the Playa
 1-4 PM
 Bombay Soleil
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>Deranged cowboy acrylic paintings by Jake Ford Wade and time capsule Salton Sea photographs by Sandi Wheaton</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Community Patchwork/
+“Reimagined Western Paintings by Jake Wade / Salton Sea Time Capsule Photographs by Sandi Wheaton”</t>
+  </si>
+  <si>
+    <t>Community Patchwork/
 Quilting Bee of the Damned
 1-2 PM
 No Shoes, Institute
-Quilting Workshop </t>
+Quilting Workshop 
+“Together we steward cast-aside fibers and create a Biennale tapestry. Sew in community, and merge tattered scraps into something new. Unlike the gods who would condemn and abandon the world they created, we explore the latent potential in each textile.“</t>
   </si>
   <si>
     <t>How to Freestyle Rap
 1:30-2:30 PM
 Sub Club
-Workshop by Rob Zeleski</t>
+Workshop by Rob Zeleski
+“Freestyle rap is rhythmic speech you discover in the moment to entertain or express yourself. A beginner friendly workshop focused on connecting to self and others.”</t>
   </si>
   <si>
     <r>
@@ -1609,43 +1489,21 @@
 (A Silicon Wasteland Production)
 by Nicholas Burrell
 3-5 PM
-Sub Club</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Only Players Left Alive
+Sub Club
+“An evening of improvised shenanigans lampooning the absurdity of startup and investment culture at the end of the world in a place of disinvestment”</t>
+  </si>
+  <si>
+    <t>Only Players Left Alive
 Post apocalyptic social simulation by Antalina Fed
 3-5:30 PM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Atlantis Inn
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>Live Action Role Play</t>
-    </r>
+Atlantis Inn
+“This is a post-apocalyptic social simulation. Playground where visitors receive new identities and enter temporary social roles. Through immersive interactions, rituals, and exchanges, participants experiment with identity, explore connection, choice, and survival.”</t>
   </si>
   <si>
     <t>Affogatos
 3-5 PM
-Drakkar Noir</t>
+Drakkar Noir
+“The night before was kind of rough, got up around 10:00, started running around looking at art had a taco at 11:00, starting to burn out and getting tired, as I raise my head the sun burning my eyes I see a line, it's affogatos”</t>
   </si>
   <si>
     <t>Judgment, Alienation, and the Constant Possibility of Being Seen
@@ -1732,26 +1590,11 @@
 Limited to 30 participants</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Charlie Chaplin Pop-Up Bar
+    <t>Charlie Chaplin Pop-Up Bar
 5-8 PM
 Bombay Bliss Beach Club
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>Roll the dice for a cocktail, mocktail, or a nosh! Electro-swing &amp; Disco with DJs Goldify and Sima&amp;Sidu</t>
-    </r>
+Roll the dice for a cocktail, mocktail, or a nosh! Electro-swing &amp; Disco with DJs Goldify and Sima&amp;Sidu
+“Sima &amp; Sidu are a DJ duo with a love for mixing South Asian rhythms and melodies into music from around the world! They are all about inspiring people to let loose and just be silly on the dance floor.”</t>
   </si>
   <si>
     <r>
@@ -1790,13 +1633,21 @@
   <si>
     <t>Prepared Tape Loops 
 6-7 PM
-Zig Zag Plaza</t>
+Zig Zag Plaza
+“A live musical performance using prepared cassette tape loops of various lengths as source material. Old Walkmans and effect pedal chains build layered, melodic sound in real time. The loops drift in and out of sync as hiss and gentle warble become part of the music.”</t>
   </si>
   <si>
     <t>Poof Alert
 6-7 PM
 Controlled Burn
-The Beach</t>
+The Beach
+"What is that thing? 
+Let's check it out. 
+A polished steel form, crawling up from the sands of the beach, a cave for you to enter. 
+Within, you see buttons! And pipes and hoses buried inside a writhing snake-like structure. 
+What is this thing?
+Press button. Fire erupts. Music happens.
+:-D"</t>
   </si>
   <si>
     <r>
@@ -1829,32 +1680,11 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t>*Cafe Bosna</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>*Cafe Bosna
 6 PM-6 AM
 Immersive Music/Coffee Experience
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t>The Estates</t>
-    </r>
+The Estates
+“An interdimensional portal to the world of ritual coffee, immersive art and global dance electronica.”</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -1877,22 +1707,26 @@
 Globalschism (The Beach)</t>
   </si>
   <si>
-    <t xml:space="preserve">EMERGENCE
+    <t>EMERGENCE
 7-8 PM
 Art Opening by Richard Wilks
-The Beach </t>
+The Beach 
+“Emergence is an other-worldly luminous sculpture experience that mysteriously started surfacing at Bombay Beach. The sculptures appear to be intelligent, organic and mechanical in form with spinal columns and finger-like limbs embracing crystal cubes. Not all have surfaced...Will more appear?”</t>
   </si>
   <si>
     <t>The Last Supper
 7-8 PM
 Controlled Burn
-The Beach</t>
+The Beach
+"This is the Last Supper before it goes up in flames. A dining table and chairs to gather around before it becomes the bonfire on which we cook our meal. Sit down, eat and enjoy, before the set itself is consumed.”</t>
   </si>
   <si>
     <t>Bacterial Beats
 by Scott (Seamus) Kildall
 7:30-8 PM
-Zig Zag Plaza</t>
+Zig Zag Plaza
+“Last year, I collected microbial samples from the Salton Sea at Bombay Beach. They produce significant electrical signals, like small batteries that vary with sunlight.
+This will be a performance where I map these into musical notes with 16 different sample jars and LEDs on each."</t>
   </si>
   <si>
     <r>
@@ -1927,16 +1761,25 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Ashes and Breath: 
+    <t>Ashes and Breath: 
 A Rite of Impermanence
 8-9 PM
-Zig Zag Plaza </t>
+Zig Zag Plaza 
+"Here, judgement is felt, not delivered.
+A sonic ritual using throat singing, ethnic instruments, fire dance, sub-bass and electronic interaction. Rooted in the ancient, oriented toward the future, the performance moves through rupture and collapse, exposing the impermanent nature of mind and matter."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S.S.S.S.S's Shared Telescope Sesh
+by Salton Sea Stellar Sky Society
+8-9 PM
+Start Sight Site, Bombay North </t>
   </si>
   <si>
     <t>Reincarnation Station
 by Suzanne Karpinski
 8-10 PM
-Institute Garden</t>
+Institute Garden
+“Welcome, wayward soul! Our condolences on your recent death. Judgement is upon you, as it is for us all. What will you take with you into your next life and what will you leave behind? The Reincarnation Station is interactive theater for 1-2 participants at a time that asks this important question.”</t>
   </si>
   <si>
     <t>ECOTECHNO 4DXYZ
@@ -1944,13 +1787,15 @@
 Red Light Theater, 
 Temple to the Scientific Method 
 Queer Shorts
-BBIFF</t>
+BBIFF
+“ECOTECHNO 4DXYZ is an immersive screening encounter that engages all seven senses to take stock of our long-negotiated relationship with and between nature and technology.“</t>
   </si>
   <si>
     <t>The Alphabet of Pleasure (Songs of Agony and Ecstasy)
 DIA LUNA
 8-9 PM
-The Ski Inn</t>
+The Ski Inn
+“The angel birds of Bombay Beach are calling you. Are you ready to fly the highest highs and dive the deepest depths of your human experience? Find sanctuary at the HEATHEN TEMPLE with music alchemists DIA LUNA. We welcome your holy wholeness! Shred your sins and sing your prayers!”</t>
   </si>
   <si>
     <r>
@@ -2075,7 +1920,8 @@
     <t>Mamacita Junior the 3rd
 8-9 PM
 The Star
-Minivan Experience with Karin</t>
+Minivan Experience with Karin
+“You are invited to experience the performance of love to Mamacita Junior the third, my tiny little minivan, which is my ever evolving home for the last 9 years.”</t>
   </si>
   <si>
     <r>
@@ -2105,15 +1951,17 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Chimaksou Presents: Ambient Atlas
+    <t>Chimaksou Presents: Ambient Atlas
 9-10 PM
-Zig Zag Plaza </t>
+Zig Zag Plaza 
+“Ambient Atlas is a traveling sound project created by Alan Kahler (chimaksou). He brings his 4-string electric bass and a table-top full of loopers, delays, reverbs, and effects to far out lands to explore the nature of time with what he calls, live and improvised site-specific sonic sculptures.”</t>
   </si>
   <si>
     <t>Everything I Desire Is Already Mine
 9-11 PM
 Temple to the Scientific Method 
-Video Installation</t>
+Video Installation
+“A 10-minute video piece featuring mud pots and manifestation, looped.”</t>
   </si>
   <si>
     <t>Karaoke
@@ -2125,7 +1973,8 @@
 Video Installation by
 Antimony Hussein
 7 PM-7 AM 
-Temple to the Scientific Method</t>
+Temple to the Scientific Method
+“Hussein, Antimony. My Niland II (Westward Journey). 2026. Video projection, multi-channel, buttermilk, car windshield, rear-view mirror. duration tbd, likely 24 hours.”</t>
   </si>
   <si>
     <r>
@@ -2186,7 +2035,124 @@
   <si>
     <t>Pickle That Up presents THE SACRAMENT OF THE HOLY BRINE
 10 PM-2 AM
-The Estates</t>
+The Estates
+"Pickle That Up brings THE SACRAMENT OF THE HOLY BRINE to all creatures great and small in Bombay Beach. 
+Witness the miracle of fermentation! 
+Visit our Altar of Acidity, receive the sacrament, and become one the faithful dill-sciples.
+If the neon pickle is glowing—come and be preserved."</t>
+  </si>
+  <si>
+    <t>Martian Takeover
+10 PM-2 AM
+Bombay Bliss Beach Club
+feat. Kiamora, Seamus &amp; Friends
+DJ performance</t>
+  </si>
+  <si>
+    <t>Party for Peace
+10 PM-2 AM
+Atlantis Inn
+Alvaro &amp; Friends on Vinyl</t>
+  </si>
+  <si>
+    <t>Willy Mason
+10-11 PM
+The Tradewinds</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Garbage Futurism: Post Waste
+UV Installation by Baer
+10 PM-2 AM
+Sotheby's
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <i/>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t>Art &amp; Music</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">*The Pussycat Lounge w/ Toledo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">11 PM-2 AM
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <i/>
+        <color theme="1"/>
+      </rPr>
+      <t>The Estates</t>
+    </r>
+  </si>
+  <si>
+    <t>Adam Freeland
+11 PM-1 AM
+Sub Club</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Bar Lescher – Nightclub Edition
+11 PM-??
+Bar Lescher, Estates
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b val="0"/>
+        <i/>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t>BYOB - Bring Your Own Boobs - Vinyls &amp; Grooves</t>
+    </r>
+  </si>
+  <si>
+    <t>Pyrotechnic Symphony
+11-11:30 PM
+Fireworks by Jonny
+The Beach
+“Multiple Firework shows &amp; dazzling effects”</t>
+  </si>
+  <si>
+    <t>Daughn Gibson
+11 PM-12 AM
+The Tradewinds</t>
+  </si>
+  <si>
+    <t>DESERT BEACH
+by TRISTAN RIO / XANDER STEENBRUGGE
+11 PM-12 AM
+PIRATESHIP (The Beach)</t>
   </si>
   <si>
     <t>Martian Takeover
@@ -2195,70 +2161,31 @@
 feat. Kiamora, Seamus &amp; Friends</t>
   </si>
   <si>
-    <t>Party for Peace
-10 PM-2 AM
-Atlantis Inn
-Alvaro &amp; Friends on Vinyl</t>
-  </si>
-  <si>
-    <t>Willy Mason
-10-11 PM
-The Tradewinds</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t xml:space="preserve">Garbage Futurism: Post Waste
-UV Installation by Baer
-10 PM-2 AM
-Sotheby's
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">*The Pussycat Lounge w/ Toledo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">11 PM-2 AM
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
         <i/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t>Art &amp; Music</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">*The Pussycat Lounge w/ Toledo
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">11 PM-2 AM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
         <color theme="1"/>
       </rPr>
       <t>The Estates</t>
     </r>
-  </si>
-  <si>
-    <t>Adam Freeland
-11 PM-1 AM
-Sub Club</t>
   </si>
   <si>
     <r>
@@ -2283,85 +2210,9 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Pyrotechnic Symphony
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>11-11:30 PM
-Fireworks by Jonny
-The Beach</t>
-    </r>
-  </si>
-  <si>
-    <t>Daughn Gibson
-11 PM-12 AM
-The Tradewinds</t>
-  </si>
-  <si>
-    <t>DESERT BEACH
-by TRISTAN RIO / XANDER STEENBRUGGE
-11 PM-12 AM
-PIRATESHIP (The Beach)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">*The Pussycat Lounge w/ Toledo
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">11 PM-2 AM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>The Estates</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t xml:space="preserve">Bar Lescher – Nightclub Edition
-11 PM-??
-Bar Lescher, Estates
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color rgb="FFFFFFFF"/>
-      </rPr>
-      <t>BYOB - Bring Your Own Boobs - Vinyls &amp; Grooves</t>
-    </r>
+    <t>Pickle That Up presents THE SACRAMENT OF THE HOLY BRINE
+10 PM-2 AM
+The Estates</t>
   </si>
   <si>
     <t>Martian Takeover
@@ -2692,13 +2543,15 @@
     <t>Precision
 1-1:30 PM
 No Shoes, Institute
-Lecture by Joel Arellano</t>
+Lecture by Joel Arellano
+“I’ll present a reading from a larger work of near-future fiction, "Precision". The work is an eschatology of the West. Tension builds as societal collapse feels imminent, but a suspicious calm challenges our assumptions of Western values, and inspire curiosity in imagined alternatives.”</t>
   </si>
   <si>
     <t>a semisensualconductor
 1:30-2 PM
 No Shoes, Institute
-Lecture by Gandala Lee</t>
+Lecture by Gandala Lee
+“As Moore's Law stopped being true in the 2020s and the US is making advanced AI chips again, a semisensualconductor explores a more organic, sensory pie experience of the latest innovations in making atomic sized transistors that power the AI race. What does it mean for a human to eat a transistor?”</t>
   </si>
   <si>
     <t>Empathy Bleed
@@ -2706,7 +2559,8 @@
 Bombay Beach Museum 
 of Bombay Beach 
 Reading by Janenne Willis
-Philosophy Conference</t>
+Philosophy Conference
+“Empathy Bleed traces two contrasting bodies of water – California’s receding Salton Sea/ancient Lake Cahuilla and the biodiverse Western Port/Wurnmarrinh in Australia – exploring the charged space in between, empathy and breath. An artist edition of the book, and a live reading with be offered.“</t>
   </si>
   <si>
     <r>
@@ -2753,7 +2607,8 @@
     <t>Endless Poetry
 3-5 PM
 The Poetry House
-Post Priori Poetry Salon</t>
+Post Priori Poetry Salon
+“The Poetry Salon is where the poets of Bombay Beach gather and offer the poems that have touched their hearts. Done entirely in silence, poetry springs forth from the most unexpected places. Bring a poem you know, or a poem you wrote.”</t>
   </si>
   <si>
     <t>Writing from the 
@@ -2766,37 +2621,47 @@
   <si>
     <t>Pharoah &amp; Tarot
 5-8 PM
-The Poetry House</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Experimental Shorts
+The Poetry House
+“Tarot Readings at The Poetry House with Pharaoh! Readings are approximately ten minutes. Pay-what-you-can, offerings are also welcome!”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">The Nest Closing Ceremony
+by Debra Berger &amp; Erica Spooner
+5-6 PM
+The Nest
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b val="0"/>
+        <i/>
+        <color theme="1"/>
+      </rPr>
+      <t>Celebrating a fiber sculpture of soft emergence.</t>
+    </r>
+  </si>
+  <si>
+    <t>Experimental Shorts
 curated by Tarcila Neves
 5-6:30 PM
 Red Light Theater, Temple to the Scientific Method
 BBIFF 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">featuring Harpazo, Ballad of Boobi Jean, Infinite Land, Buzzkill, Fall in Love with Death, Mountains of the Moon, Manifesto Antropofago 2.0, Falling into Language, We might be dead by tomorrow, let's love today, Turao on Mars, The Classical Reunion, Wedding of the Sun and Moon, Ginostra Monstro </t>
-    </r>
+featuring Harpazo, Ballad of Boobi Jean, Infinite Land, Buzzkill, Fall in Love with Death, Mountains of the Moon, Manifesto Antropofago 2.0, Falling into Language, We might be dead by tomorrow, let's love today, Turao on Mars, The Classical Reunion, Wedding of the Sun and Moon, Ginostra Monstro 
+“A surreal, seriocomic narrative short film about fear, judgement, the lust for death, and queer friendship at the end of the world. A tenacious and ultimately hopeful film debut shot in Bombay Beach under the Buck Moon of 2023, only growing more relevant with each tick of the doomsday clock.”</t>
   </si>
   <si>
     <t>Olive
 6-7 PM
 Zig Zag Plaza
-Performance by Nora Dell</t>
+Performance by Nora Dell
+“I participate in the BBB as a giant olive, letting the elements, environment, and other artists change and influence me. Over the course of the weekend, I devise/create a final performance, and perform it at midnight on Sunday.”</t>
   </si>
   <si>
     <r>
@@ -2837,29 +2702,22 @@
     <t>Lost Chord Divine
 6:30-7:30 PM
 Henderson Hall
-Beverly Kitty Green</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Ann-Marie Lindblad Performs!
+Beverly Kitty Green
+"I sought but to seek it vainly, 
+that one lost chord divine; 
+which came from the soul of the organ, 
+and entered into mine. 
+It may be that death's bright angel
+Will speak in that chord again,
+It may be that only in Heaven
+I shall hear that grand Amen.”</t>
+  </si>
+  <si>
+    <t>Ann-Marie Lindblad Performs!
 7-8 PM
 Zig Zag Plaza
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b val="0"/>
-        <i/>
-        <color theme="1"/>
-      </rPr>
-      <t>A lo-fi, feral, shape-shifting hour of live music, clown-esque performance art, poetry, soundscapes, and rubber chicken orchestra.</t>
-    </r>
+"Live music. Interruptions. Clown. 
+Joy gets thrown away. The desert listens."</t>
   </si>
   <si>
     <r>
@@ -2897,7 +2755,8 @@
 By Douglass Clarke
 Directed by Cameron Gregg
 8-8:30 PM
-Zig Zag Plaza</t>
+Zig Zag Plaza
+“What would you do if providence found its way into your life after years of struggle. What if the people in your life finally contained traits that matched your ideals. What if one day you discovered that all your dreams were set to come true as you're surrounded by those near and dear to you?”</t>
   </si>
   <si>
     <t>The Last Canter
@@ -2913,13 +2772,15 @@
 8-10 PM
 Red Light Theater, Temple to the Scientific Method
 Documentary Feature
-BBIFF</t>
+BBIFF
+“The Colorado, narrated by the stage legend Marc Rylance, takes us on an epic journey through the prehistoric settlements of the region, the period of European exploration, the dam-building era, modern industrial agriculture and immigration, and the impact of climate change.”</t>
   </si>
   <si>
     <t>Eat Pray Cult
 8:30-9:30 PM
 Zig Zag Plaza
-Comedy Performance by Amy Brown Carver</t>
+Comedy Performance by Amy Brown Carver
+“What would it take for you to leave your comfortable life? Join Amy Brown Carver for 45-minutes of stand-up and collective comedy adventure about one woman’s search for freedom, meaning, and the closest flush toilet.“</t>
   </si>
   <si>
     <t>Name</t>
@@ -3491,7 +3352,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="169">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3656,9 +3517,6 @@
     <xf borderId="5" fillId="0" fontId="17" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="7" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -3765,6 +3623,9 @@
     <xf borderId="4" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="14" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -3856,7 +3717,7 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="11" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="15" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -3903,6 +3764,9 @@
     <xf borderId="0" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="5" fillId="11" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="15" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -3923,6 +3787,9 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="14" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="10" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -3987,7 +3854,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Dane Sandborg" id="{86379b4e-de9c-4987-864f-db4cceedcc00}" providerId="google-sheets"/>
+  <x18tc:person displayName="Dane Sandborg" id="{50309944-cabd-4666-9d27-db34fd7bf39c}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -4187,7 +4054,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D53" dT="2026-03-23T19:38:09.00" personId="{86379b4e-de9c-4987-864f-db4cceedcc00}" id="{dbc866ff-36c2-4b34-a443-fd7ab61a53ab}" done="0">
+  <x18tc:threadedComment ref="D53" dT="2026-03-23T19:38:09.00" personId="{50309944-cabd-4666-9d27-db34fd7bf39c}" id="{1a9a9bfc-57a7-4d31-a9a1-1f06d07d8acf}" done="0">
     <x18tc:text xml:space="preserve">The lost soul train</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -4738,16 +4605,13 @@
       <c r="B51" s="57">
         <v>0.7916666666666666</v>
       </c>
-      <c r="D51" s="58" t="s">
-        <v>29</v>
-      </c>
+      <c r="D51" s="38"/>
       <c r="E51" s="40"/>
     </row>
     <row r="52" ht="48.0" customHeight="1">
       <c r="A52" s="21"/>
       <c r="B52" s="40"/>
       <c r="C52" s="55"/>
-      <c r="D52" s="41"/>
       <c r="E52" s="40"/>
     </row>
     <row r="53" ht="48.75" customHeight="1">
@@ -4755,21 +4619,21 @@
       <c r="B53" s="48">
         <v>0.8333333333333334</v>
       </c>
-      <c r="C53" s="59" t="s">
+      <c r="C53" s="58" t="s">
+        <v>29</v>
+      </c>
+      <c r="D53" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="D53" s="56" t="s">
+      <c r="E53" s="40"/>
+      <c r="G53" s="59" t="s">
         <v>31</v>
-      </c>
-      <c r="E53" s="40"/>
-      <c r="G53" s="60" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="54" ht="23.25" customHeight="1">
       <c r="A54" s="21"/>
       <c r="B54" s="17"/>
-      <c r="C54" s="61"/>
+      <c r="C54" s="60"/>
       <c r="D54" s="41"/>
       <c r="E54" s="40"/>
       <c r="G54" s="40"/>
@@ -4779,15 +4643,15 @@
       <c r="B55" s="44">
         <v>0.875</v>
       </c>
-      <c r="C55" s="62"/>
-      <c r="D55" s="63" t="s">
+      <c r="C55" s="61"/>
+      <c r="D55" s="62" t="s">
+        <v>32</v>
+      </c>
+      <c r="E55" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="E55" s="46" t="s">
+      <c r="F55" s="63" t="s">
         <v>34</v>
-      </c>
-      <c r="F55" s="64" t="s">
-        <v>35</v>
       </c>
       <c r="G55" s="40"/>
     </row>
@@ -4798,7 +4662,7 @@
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="56" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E56" s="41"/>
       <c r="F56" s="45"/>
@@ -4817,47 +4681,47 @@
     </row>
     <row r="58" ht="19.5" customHeight="1">
       <c r="A58" s="21"/>
-      <c r="B58" s="65">
+      <c r="B58" s="64">
         <v>0.0</v>
       </c>
-      <c r="C58" s="66"/>
+      <c r="C58" s="65"/>
       <c r="D58" s="41"/>
       <c r="F58" s="41"/>
       <c r="G58" s="41"/>
     </row>
     <row r="59">
       <c r="A59" s="21"/>
-      <c r="B59" s="67" t="s">
-        <v>37</v>
-      </c>
-      <c r="C59" s="68"/>
-      <c r="D59" s="69"/>
-      <c r="E59" s="70"/>
-      <c r="F59" s="70"/>
-      <c r="G59" s="71"/>
-      <c r="H59" s="71"/>
-      <c r="I59" s="71"/>
-      <c r="J59" s="71"/>
-      <c r="K59" s="71"/>
-      <c r="L59" s="71"/>
-      <c r="M59" s="71"/>
-      <c r="N59" s="71"/>
-      <c r="O59" s="72"/>
-      <c r="P59" s="72"/>
+      <c r="B59" s="66" t="s">
+        <v>36</v>
+      </c>
+      <c r="C59" s="67"/>
+      <c r="D59" s="68"/>
+      <c r="E59" s="69"/>
+      <c r="F59" s="69"/>
+      <c r="G59" s="70"/>
+      <c r="H59" s="70"/>
+      <c r="I59" s="70"/>
+      <c r="J59" s="70"/>
+      <c r="K59" s="70"/>
+      <c r="L59" s="70"/>
+      <c r="M59" s="70"/>
+      <c r="N59" s="70"/>
+      <c r="O59" s="71"/>
+      <c r="P59" s="71"/>
     </row>
     <row r="60" ht="28.5" customHeight="1">
       <c r="A60" s="21"/>
-      <c r="B60" s="73">
+      <c r="B60" s="72">
         <v>0.3333333333333333</v>
       </c>
       <c r="C60" s="31"/>
       <c r="D60" s="31"/>
       <c r="E60" s="31"/>
       <c r="F60" s="56" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G60" s="38"/>
-      <c r="H60" s="74"/>
+      <c r="H60" s="73"/>
       <c r="I60" s="31"/>
       <c r="J60" s="31"/>
       <c r="K60" s="31"/>
@@ -4869,78 +4733,78 @@
     </row>
     <row r="61" ht="30.0" customHeight="1">
       <c r="A61" s="21"/>
-      <c r="B61" s="73">
+      <c r="B61" s="72">
         <v>0.375</v>
       </c>
-      <c r="C61" s="75"/>
+      <c r="C61" s="74"/>
       <c r="F61" s="40"/>
-      <c r="H61" s="76"/>
+      <c r="H61" s="75"/>
     </row>
     <row r="62" ht="71.25" customHeight="1">
       <c r="A62" s="21"/>
-      <c r="B62" s="77">
+      <c r="B62" s="76">
         <v>0.4166666666666667</v>
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="E62" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="E62" s="64" t="s">
-        <v>40</v>
-      </c>
       <c r="F62" s="40"/>
-      <c r="H62" s="76"/>
+      <c r="H62" s="75"/>
     </row>
     <row r="63" ht="71.25" customHeight="1">
       <c r="A63" s="21"/>
-      <c r="B63" s="77"/>
+      <c r="B63" s="76"/>
       <c r="C63" s="17"/>
       <c r="D63" s="40"/>
-      <c r="E63" s="78"/>
+      <c r="E63" s="77"/>
       <c r="F63" s="40"/>
-      <c r="H63" s="76"/>
+      <c r="H63" s="75"/>
     </row>
     <row r="64" ht="55.5" customHeight="1">
       <c r="A64" s="21"/>
-      <c r="B64" s="77">
+      <c r="B64" s="76">
         <v>0.4583333333333333</v>
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E64" s="30" t="s">
         <v>41</v>
-      </c>
-      <c r="E64" s="30" t="s">
-        <v>42</v>
       </c>
       <c r="F64" s="40"/>
       <c r="G64" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="H64" s="76"/>
+        <v>42</v>
+      </c>
+      <c r="H64" s="75"/>
     </row>
     <row r="65" ht="25.5" customHeight="1">
       <c r="A65" s="21"/>
-      <c r="B65" s="77"/>
-      <c r="C65" s="75"/>
+      <c r="B65" s="76"/>
+      <c r="C65" s="74"/>
       <c r="D65" s="40"/>
       <c r="E65" s="40"/>
       <c r="F65" s="40"/>
       <c r="G65" s="41"/>
-      <c r="H65" s="76"/>
+      <c r="H65" s="75"/>
     </row>
     <row r="66" ht="27.75" customHeight="1">
       <c r="A66" s="21"/>
-      <c r="B66" s="79">
+      <c r="B66" s="78">
         <v>0.5</v>
       </c>
-      <c r="C66" s="80" t="s">
-        <v>44</v>
+      <c r="C66" s="79" t="s">
+        <v>43</v>
       </c>
       <c r="D66" s="40"/>
       <c r="E66" s="40"/>
       <c r="F66" s="40"/>
       <c r="G66" s="38"/>
-      <c r="H66" s="76"/>
+      <c r="H66" s="75"/>
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="21"/>
@@ -4949,58 +4813,58 @@
       <c r="D67" s="40"/>
       <c r="E67" s="41"/>
       <c r="F67" s="40"/>
-      <c r="H67" s="76"/>
+      <c r="H67" s="75"/>
     </row>
     <row r="68" ht="46.5" customHeight="1">
       <c r="A68" s="21"/>
-      <c r="B68" s="79">
+      <c r="B68" s="78">
         <v>0.5416666666666666</v>
       </c>
       <c r="C68" s="41"/>
       <c r="D68" s="41"/>
       <c r="E68" s="31"/>
       <c r="F68" s="41"/>
-      <c r="H68" s="76"/>
+      <c r="H68" s="75"/>
     </row>
     <row r="69" ht="64.5" customHeight="1">
       <c r="A69" s="21"/>
-      <c r="B69" s="77">
+      <c r="B69" s="76">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C69" s="81"/>
+      <c r="C69" s="80"/>
       <c r="D69" s="31"/>
-      <c r="E69" s="82" t="s">
+      <c r="E69" s="81" t="s">
+        <v>44</v>
+      </c>
+      <c r="F69" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="F69" s="30" t="s">
+      <c r="H69" s="75"/>
+      <c r="N69" s="37" t="s">
         <v>46</v>
-      </c>
-      <c r="H69" s="76"/>
-      <c r="N69" s="37" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="70" ht="33.75" customHeight="1">
       <c r="A70" s="21"/>
       <c r="B70" s="40"/>
       <c r="C70" s="40"/>
-      <c r="E70" s="66"/>
+      <c r="E70" s="65"/>
       <c r="F70" s="40"/>
-      <c r="H70" s="76"/>
+      <c r="H70" s="75"/>
       <c r="N70" s="40"/>
     </row>
     <row r="71" ht="47.25" customHeight="1">
       <c r="A71" s="21"/>
-      <c r="B71" s="77">
+      <c r="B71" s="76">
         <v>0.625</v>
       </c>
       <c r="C71" s="40"/>
       <c r="E71" s="31"/>
       <c r="F71" s="40"/>
       <c r="G71" s="56" t="s">
-        <v>48</v>
-      </c>
-      <c r="H71" s="76"/>
+        <v>47</v>
+      </c>
+      <c r="H71" s="75"/>
       <c r="N71" s="40"/>
     </row>
     <row r="72" ht="53.25" customHeight="1">
@@ -5009,62 +4873,62 @@
       <c r="C72" s="40"/>
       <c r="F72" s="41"/>
       <c r="G72" s="40"/>
-      <c r="H72" s="76"/>
+      <c r="H72" s="75"/>
       <c r="N72" s="40"/>
     </row>
     <row r="73" ht="39.0" customHeight="1">
       <c r="A73" s="21"/>
-      <c r="B73" s="77">
+      <c r="B73" s="76">
         <v>0.6666666666666666</v>
       </c>
       <c r="C73" s="40"/>
-      <c r="D73" s="83" t="s">
+      <c r="D73" s="82" t="s">
+        <v>48</v>
+      </c>
+      <c r="E73" s="81" t="s">
         <v>49</v>
       </c>
-      <c r="E73" s="82" t="s">
+      <c r="F73" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="F73" s="56" t="s">
-        <v>51</v>
-      </c>
       <c r="G73" s="40"/>
-      <c r="H73" s="76"/>
+      <c r="H73" s="75"/>
       <c r="N73" s="40"/>
     </row>
     <row r="74" ht="64.5" customHeight="1">
       <c r="A74" s="21"/>
-      <c r="B74" s="84"/>
+      <c r="B74" s="83"/>
       <c r="C74" s="40"/>
       <c r="D74" s="40"/>
       <c r="E74" s="17"/>
       <c r="F74" s="41"/>
       <c r="G74" s="40"/>
-      <c r="H74" s="76"/>
-      <c r="I74" s="85" t="s">
-        <v>52</v>
+      <c r="H74" s="75"/>
+      <c r="I74" s="84" t="s">
+        <v>51</v>
       </c>
       <c r="N74" s="41"/>
     </row>
     <row r="75" ht="56.25" customHeight="1">
       <c r="A75" s="21"/>
-      <c r="B75" s="79">
+      <c r="B75" s="78">
         <v>0.7083333333333334</v>
       </c>
       <c r="C75" s="40"/>
-      <c r="D75" s="83" t="s">
+      <c r="D75" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="E75" s="17"/>
+      <c r="F75" s="85"/>
+      <c r="G75" s="86" t="s">
         <v>53</v>
       </c>
-      <c r="E75" s="17"/>
-      <c r="F75" s="86"/>
-      <c r="G75" s="87" t="s">
+      <c r="H75" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="H75" s="85" t="s">
+      <c r="I75" s="75"/>
+      <c r="N75" s="37" t="s">
         <v>55</v>
-      </c>
-      <c r="I75" s="76"/>
-      <c r="N75" s="37" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="76" ht="57.75" customHeight="1">
@@ -5074,17 +4938,17 @@
       <c r="D76" s="40"/>
       <c r="E76" s="17"/>
       <c r="F76" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="G76" s="40"/>
+      <c r="H76" s="75"/>
+      <c r="I76" s="87"/>
+      <c r="K76" s="88" t="s">
         <v>57</v>
       </c>
-      <c r="G76" s="40"/>
-      <c r="H76" s="76"/>
-      <c r="I76" s="88"/>
-      <c r="K76" s="89" t="s">
+      <c r="N76" s="40"/>
+      <c r="P76" s="89" t="s">
         <v>58</v>
-      </c>
-      <c r="N76" s="40"/>
-      <c r="P76" s="90" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="77" ht="76.5" customHeight="1">
@@ -5093,24 +4957,24 @@
         <v>0.75</v>
       </c>
       <c r="C77" s="40"/>
-      <c r="D77" s="91"/>
+      <c r="D77" s="90"/>
       <c r="E77" s="17"/>
       <c r="F77" s="40"/>
       <c r="G77" s="40"/>
-      <c r="H77" s="76"/>
-      <c r="I77" s="92" t="s">
+      <c r="H77" s="75"/>
+      <c r="I77" s="91" t="s">
+        <v>59</v>
+      </c>
+      <c r="J77" s="92" t="s">
         <v>60</v>
       </c>
-      <c r="J77" s="93" t="s">
+      <c r="K77" s="40"/>
+      <c r="L77" s="63" t="s">
         <v>61</v>
-      </c>
-      <c r="K77" s="40"/>
-      <c r="L77" s="64" t="s">
-        <v>62</v>
       </c>
       <c r="N77" s="40"/>
       <c r="O77" s="33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P77" s="40"/>
     </row>
@@ -5118,16 +4982,16 @@
       <c r="A78" s="21"/>
       <c r="B78" s="40"/>
       <c r="C78" s="40"/>
-      <c r="D78" s="88"/>
+      <c r="D78" s="87"/>
       <c r="E78" s="17"/>
       <c r="F78" s="41"/>
       <c r="G78" s="41"/>
-      <c r="H78" s="88"/>
+      <c r="H78" s="87"/>
       <c r="I78" s="40"/>
       <c r="J78" s="40"/>
       <c r="K78" s="40"/>
       <c r="L78" s="30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N78" s="40"/>
       <c r="O78" s="40"/>
@@ -5135,29 +4999,29 @@
     </row>
     <row r="79" ht="33.75" customHeight="1">
       <c r="A79" s="21"/>
-      <c r="B79" s="94">
+      <c r="B79" s="93">
         <v>0.7916666666666666</v>
       </c>
       <c r="C79" s="40"/>
       <c r="D79" s="56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E79" s="17"/>
       <c r="F79" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="G79" s="94" t="s">
         <v>66</v>
       </c>
-      <c r="G79" s="95" t="s">
+      <c r="H79" s="95" t="s">
         <v>67</v>
-      </c>
-      <c r="H79" s="96" t="s">
-        <v>68</v>
       </c>
       <c r="I79" s="40"/>
       <c r="J79" s="40"/>
       <c r="K79" s="41"/>
       <c r="L79" s="40"/>
       <c r="M79" s="56" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N79" s="40"/>
       <c r="O79" s="40"/>
@@ -5168,15 +5032,15 @@
       <c r="B80" s="17"/>
       <c r="C80" s="40"/>
       <c r="D80" s="40"/>
-      <c r="E80" s="58" t="s">
-        <v>70</v>
+      <c r="E80" s="96" t="s">
+        <v>69</v>
       </c>
       <c r="F80" s="41"/>
       <c r="H80" s="40"/>
       <c r="I80" s="41"/>
       <c r="J80" s="41"/>
       <c r="K80" s="30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L80" s="40"/>
       <c r="M80" s="40"/>
@@ -5189,29 +5053,29 @@
       <c r="B81" s="97">
         <v>0.8333333333333334</v>
       </c>
-      <c r="C81" s="80" t="s">
-        <v>72</v>
+      <c r="C81" s="79" t="s">
+        <v>71</v>
       </c>
       <c r="D81" s="40"/>
       <c r="E81" s="40"/>
       <c r="F81" s="98" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H81" s="40"/>
       <c r="I81" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="J81" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="J81" s="99" t="s">
-        <v>75</v>
-      </c>
       <c r="K81" s="30" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="L81" s="40"/>
       <c r="M81" s="40"/>
       <c r="N81" s="40"/>
       <c r="O81" s="56" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P81" s="40"/>
     </row>
@@ -5238,22 +5102,22 @@
         <v>0.875</v>
       </c>
       <c r="C83" s="41"/>
-      <c r="E83" s="95" t="s">
-        <v>78</v>
+      <c r="E83" s="94" t="s">
+        <v>76</v>
       </c>
       <c r="F83" s="40"/>
       <c r="G83" s="100" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H83" s="30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I83" s="45"/>
       <c r="J83" s="40"/>
       <c r="K83" s="40"/>
       <c r="L83" s="40"/>
       <c r="M83" s="101" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="N83" s="40"/>
       <c r="O83" s="40"/>
@@ -5263,14 +5127,14 @@
       <c r="A84" s="21"/>
       <c r="B84" s="17"/>
       <c r="C84" s="18"/>
-      <c r="D84" s="58" t="s">
-        <v>82</v>
+      <c r="D84" s="96" t="s">
+        <v>80</v>
       </c>
       <c r="F84" s="40"/>
       <c r="G84" s="40"/>
       <c r="H84" s="41"/>
       <c r="I84" s="102" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J84" s="41"/>
       <c r="K84" s="40"/>
@@ -5288,22 +5152,22 @@
       <c r="C85" s="103"/>
       <c r="D85" s="38"/>
       <c r="F85" s="104" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G85" s="40"/>
       <c r="H85" s="105"/>
       <c r="I85" s="40"/>
       <c r="J85" s="56" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K85" s="40"/>
       <c r="L85" s="106" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M85" s="40"/>
       <c r="N85" s="40"/>
       <c r="O85" s="99" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P85" s="40"/>
     </row>
@@ -5326,29 +5190,29 @@
         <v>0.9583333333333334</v>
       </c>
       <c r="D87" s="107" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F87" s="17"/>
       <c r="G87" s="40"/>
       <c r="I87" s="40"/>
       <c r="J87" s="40"/>
       <c r="K87" s="40"/>
-      <c r="M87" s="95" t="s">
-        <v>88</v>
-      </c>
-      <c r="N87" s="95" t="s">
-        <v>89</v>
+      <c r="M87" s="94" t="s">
+        <v>86</v>
+      </c>
+      <c r="N87" s="94" t="s">
+        <v>87</v>
       </c>
       <c r="O87" s="40"/>
       <c r="P87" s="40"/>
     </row>
     <row r="88" ht="87.0" customHeight="1">
       <c r="A88" s="21"/>
-      <c r="B88" s="66"/>
-      <c r="E88" s="95" t="s">
-        <v>90</v>
-      </c>
-      <c r="F88" s="66"/>
+      <c r="B88" s="65"/>
+      <c r="E88" s="94" t="s">
+        <v>88</v>
+      </c>
+      <c r="F88" s="65"/>
       <c r="G88" s="41"/>
       <c r="I88" s="41"/>
       <c r="J88" s="41"/>
@@ -5359,7 +5223,7 @@
     <row r="89">
       <c r="A89" s="21"/>
       <c r="B89" s="108" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C89" s="109"/>
       <c r="E89" s="110"/>
@@ -5377,44 +5241,44 @@
     </row>
     <row r="90" ht="77.25" customHeight="1">
       <c r="A90" s="21"/>
-      <c r="B90" s="79">
+      <c r="B90" s="78">
         <v>1.0</v>
       </c>
       <c r="C90" s="111"/>
       <c r="D90" s="38"/>
-      <c r="E90" s="95" t="s">
+      <c r="E90" s="94" t="s">
+        <v>88</v>
+      </c>
+      <c r="F90" s="94" t="s">
         <v>90</v>
       </c>
-      <c r="F90" s="95" t="s">
+      <c r="G90" s="100" t="s">
+        <v>91</v>
+      </c>
+      <c r="H90" s="105"/>
+      <c r="I90" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="G90" s="100" t="s">
+      <c r="J90" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="K90" s="100" t="s">
         <v>93</v>
       </c>
-      <c r="H90" s="105"/>
-      <c r="I90" s="95" t="s">
+      <c r="L90" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="M90" s="94" t="s">
+        <v>86</v>
+      </c>
+      <c r="N90" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="J90" s="56" t="s">
-        <v>85</v>
-      </c>
-      <c r="K90" s="100" t="s">
-        <v>95</v>
-      </c>
-      <c r="L90" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="M90" s="95" t="s">
-        <v>88</v>
-      </c>
-      <c r="N90" s="95" t="s">
-        <v>96</v>
-      </c>
       <c r="O90" s="99" t="s">
-        <v>75</v>
-      </c>
-      <c r="P90" s="90" t="s">
-        <v>59</v>
+        <v>74</v>
+      </c>
+      <c r="P90" s="89" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="91" ht="30.0" customHeight="1">
@@ -5422,7 +5286,7 @@
       <c r="B91" s="40"/>
       <c r="C91" s="40"/>
       <c r="D91" s="112" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G91" s="40"/>
       <c r="J91" s="40"/>
@@ -5433,7 +5297,7 @@
     </row>
     <row r="92" ht="45.0" customHeight="1">
       <c r="A92" s="21"/>
-      <c r="B92" s="79">
+      <c r="B92" s="78">
         <v>0.041666666666666664</v>
       </c>
       <c r="C92" s="40"/>
@@ -5447,7 +5311,7 @@
     </row>
     <row r="93" ht="40.5" customHeight="1">
       <c r="A93" s="21"/>
-      <c r="B93" s="79"/>
+      <c r="B93" s="78"/>
       <c r="C93" s="40"/>
       <c r="D93" s="40"/>
       <c r="G93" s="41"/>
@@ -5459,7 +5323,7 @@
     </row>
     <row r="94" ht="21.0" customHeight="1">
       <c r="A94" s="21"/>
-      <c r="B94" s="79">
+      <c r="B94" s="78">
         <v>0.08333333333333333</v>
       </c>
       <c r="C94" s="40"/>
@@ -5475,18 +5339,18 @@
     </row>
     <row r="95" ht="21.0" customHeight="1">
       <c r="A95" s="21"/>
-      <c r="B95" s="79"/>
+      <c r="B95" s="78"/>
       <c r="C95" s="40"/>
       <c r="D95" s="38"/>
       <c r="K95" s="40"/>
-      <c r="M95" s="95"/>
-      <c r="N95" s="95"/>
+      <c r="M95" s="94"/>
+      <c r="N95" s="94"/>
       <c r="O95" s="40"/>
       <c r="P95" s="40"/>
     </row>
     <row r="96" ht="16.5" customHeight="1">
       <c r="A96" s="21"/>
-      <c r="B96" s="79">
+      <c r="B96" s="78">
         <v>0.125</v>
       </c>
       <c r="C96" s="40"/>
@@ -5499,7 +5363,7 @@
     </row>
     <row r="97">
       <c r="A97" s="21"/>
-      <c r="B97" s="79">
+      <c r="B97" s="78">
         <v>0.16666666666666666</v>
       </c>
       <c r="C97" s="40"/>
@@ -5509,7 +5373,7 @@
     </row>
     <row r="98">
       <c r="A98" s="21"/>
-      <c r="B98" s="79">
+      <c r="B98" s="78">
         <v>0.20833333333333334</v>
       </c>
       <c r="C98" s="40"/>
@@ -5519,7 +5383,7 @@
     </row>
     <row r="99">
       <c r="A99" s="21"/>
-      <c r="B99" s="77">
+      <c r="B99" s="76">
         <v>0.25</v>
       </c>
       <c r="C99" s="40"/>
@@ -5529,7 +5393,7 @@
     </row>
     <row r="100" ht="21.0" customHeight="1">
       <c r="A100" s="21"/>
-      <c r="B100" s="79">
+      <c r="B100" s="78">
         <v>0.2916666666666667</v>
       </c>
       <c r="C100" s="40"/>
@@ -5539,27 +5403,27 @@
     </row>
     <row r="101" ht="18.75" customHeight="1">
       <c r="A101" s="21"/>
-      <c r="B101" s="79">
+      <c r="B101" s="78">
         <v>0.3333333333333333</v>
       </c>
       <c r="C101" s="40"/>
       <c r="J101" s="56" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="K101" s="40"/>
       <c r="O101" s="37" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P101" s="116"/>
     </row>
     <row r="102" ht="111.0" customHeight="1">
       <c r="A102" s="21"/>
-      <c r="B102" s="79">
+      <c r="B102" s="78">
         <v>0.375</v>
       </c>
       <c r="C102" s="40"/>
-      <c r="D102" s="64" t="s">
-        <v>99</v>
+      <c r="D102" s="63" t="s">
+        <v>98</v>
       </c>
       <c r="J102" s="40"/>
       <c r="K102" s="40"/>
@@ -5568,21 +5432,21 @@
     </row>
     <row r="103" ht="61.5" customHeight="1">
       <c r="A103" s="21"/>
-      <c r="B103" s="79">
+      <c r="B103" s="78">
         <v>0.4166666666666667</v>
       </c>
       <c r="C103" s="40"/>
-      <c r="D103" s="83" t="s">
+      <c r="D103" s="82" t="s">
+        <v>99</v>
+      </c>
+      <c r="E103" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="F103" s="86" t="s">
         <v>100</v>
       </c>
-      <c r="E103" s="64" t="s">
-        <v>40</v>
-      </c>
-      <c r="F103" s="87" t="s">
+      <c r="H103" s="30" t="s">
         <v>101</v>
-      </c>
-      <c r="H103" s="30" t="s">
-        <v>102</v>
       </c>
       <c r="J103" s="40"/>
       <c r="K103" s="40"/>
@@ -5595,10 +5459,10 @@
       <c r="C104" s="40"/>
       <c r="D104" s="40"/>
       <c r="E104" s="117" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F104" s="41"/>
-      <c r="G104" s="69"/>
+      <c r="G104" s="68"/>
       <c r="H104" s="41"/>
       <c r="J104" s="40"/>
       <c r="K104" s="40"/>
@@ -5607,22 +5471,22 @@
     </row>
     <row r="105" ht="52.5" customHeight="1">
       <c r="A105" s="21"/>
-      <c r="B105" s="79">
+      <c r="B105" s="78">
         <v>0.4583333333333333</v>
       </c>
       <c r="C105" s="40"/>
-      <c r="D105" s="83" t="s">
-        <v>104</v>
+      <c r="D105" s="82" t="s">
+        <v>103</v>
       </c>
       <c r="E105" s="38"/>
       <c r="F105" s="118" t="s">
+        <v>104</v>
+      </c>
+      <c r="G105" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="G105" s="99" t="s">
+      <c r="H105" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="H105" s="30" t="s">
-        <v>42</v>
       </c>
       <c r="I105" s="37" t="s">
         <v>107</v>
@@ -5655,11 +5519,11 @@
     </row>
     <row r="107" ht="33.0" customHeight="1">
       <c r="A107" s="21"/>
-      <c r="B107" s="79">
+      <c r="B107" s="78">
         <v>0.5</v>
       </c>
       <c r="C107" s="40"/>
-      <c r="D107" s="83" t="s">
+      <c r="D107" s="82" t="s">
         <v>110</v>
       </c>
       <c r="E107" s="41"/>
@@ -5698,10 +5562,10 @@
       <c r="B109" s="97">
         <v>0.5416666666666666</v>
       </c>
-      <c r="C109" s="80" t="s">
+      <c r="C109" s="79" t="s">
         <v>113</v>
       </c>
-      <c r="D109" s="83" t="s">
+      <c r="D109" s="82" t="s">
         <v>114</v>
       </c>
       <c r="E109" s="120" t="s">
@@ -5780,11 +5644,11 @@
     </row>
     <row r="113" ht="66.75" customHeight="1">
       <c r="A113" s="21"/>
-      <c r="B113" s="94">
+      <c r="B113" s="93">
         <v>0.625</v>
       </c>
       <c r="C113" s="122"/>
-      <c r="D113" s="83" t="s">
+      <c r="D113" s="82" t="s">
         <v>121</v>
       </c>
       <c r="E113" s="41"/>
@@ -5807,11 +5671,11 @@
     </row>
     <row r="114" ht="43.5" customHeight="1">
       <c r="A114" s="21"/>
-      <c r="B114" s="79">
+      <c r="B114" s="78">
         <v>0.6666666666666666</v>
       </c>
       <c r="C114" s="17"/>
-      <c r="D114" s="83" t="s">
+      <c r="D114" s="82" t="s">
         <v>125</v>
       </c>
       <c r="E114" s="56" t="s">
@@ -5851,7 +5715,7 @@
     </row>
     <row r="116" ht="57.75" customHeight="1">
       <c r="A116" s="21"/>
-      <c r="B116" s="77">
+      <c r="B116" s="76">
         <v>0.7083333333333334</v>
       </c>
       <c r="C116" s="17"/>
@@ -5861,7 +5725,7 @@
       <c r="E116" s="41"/>
       <c r="F116" s="40"/>
       <c r="G116" s="30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H116" s="41"/>
       <c r="I116" s="118" t="s">
@@ -5881,7 +5745,7 @@
       <c r="B117" s="40"/>
       <c r="C117" s="17"/>
       <c r="D117" s="41"/>
-      <c r="E117" s="64" t="s">
+      <c r="E117" s="63" t="s">
         <v>132</v>
       </c>
       <c r="F117" s="40"/>
@@ -5917,10 +5781,10 @@
       </c>
       <c r="K118" s="113"/>
       <c r="L118" s="30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M118" s="33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N118" s="40"/>
       <c r="O118" s="40"/>
@@ -5948,18 +5812,18 @@
     </row>
     <row r="120" ht="62.25" customHeight="1">
       <c r="A120" s="21"/>
-      <c r="B120" s="77">
+      <c r="B120" s="76">
         <v>0.7916666666666666</v>
       </c>
       <c r="C120" s="17"/>
-      <c r="D120" s="83" t="s">
+      <c r="D120" s="82" t="s">
         <v>138</v>
       </c>
       <c r="E120" s="30" t="s">
         <v>139</v>
       </c>
       <c r="F120" s="40"/>
-      <c r="G120" s="95" t="s">
+      <c r="G120" s="94" t="s">
         <v>140</v>
       </c>
       <c r="H120" s="56" t="s">
@@ -5973,7 +5837,7 @@
       <c r="L120" s="40"/>
       <c r="M120" s="40"/>
       <c r="N120" s="56" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="O120" s="40"/>
       <c r="P120" s="40"/>
@@ -5999,10 +5863,10 @@
     </row>
     <row r="122" ht="80.25" customHeight="1">
       <c r="A122" s="21"/>
-      <c r="B122" s="79">
+      <c r="B122" s="78">
         <v>0.8333333333333334</v>
       </c>
-      <c r="C122" s="80" t="s">
+      <c r="C122" s="79" t="s">
         <v>144</v>
       </c>
       <c r="D122" s="40"/>
@@ -6010,28 +5874,28 @@
         <v>145</v>
       </c>
       <c r="F122" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="H122" s="58" t="s">
         <v>146</v>
       </c>
+      <c r="H122" s="96" t="s">
+        <v>147</v>
+      </c>
       <c r="I122" s="46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J122" s="126" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K122" s="118" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L122" s="56" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="M122" s="126" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="N122" s="56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O122" s="40"/>
       <c r="P122" s="40"/>
@@ -6043,8 +5907,8 @@
       <c r="D123" s="41"/>
       <c r="E123" s="40"/>
       <c r="F123" s="40"/>
-      <c r="G123" s="87" t="s">
-        <v>153</v>
+      <c r="G123" s="86" t="s">
+        <v>154</v>
       </c>
       <c r="H123" s="40"/>
       <c r="I123" s="41"/>
@@ -6058,15 +5922,15 @@
     </row>
     <row r="124" ht="82.5" customHeight="1">
       <c r="A124" s="21"/>
-      <c r="B124" s="79">
+      <c r="B124" s="78">
         <v>0.875</v>
       </c>
       <c r="C124" s="41"/>
       <c r="D124" s="121" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E124" s="125" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F124" s="30" t="s">
         <v>127</v>
@@ -6074,24 +5938,24 @@
       <c r="G124" s="41"/>
       <c r="H124" s="41"/>
       <c r="I124" s="46" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J124" s="30" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K124" s="40"/>
       <c r="L124" s="40"/>
       <c r="M124" s="38"/>
-      <c r="N124" s="89" t="s">
-        <v>158</v>
+      <c r="N124" s="88" t="s">
+        <v>159</v>
       </c>
       <c r="O124" s="40"/>
       <c r="P124" s="40"/>
     </row>
     <row r="125" ht="86.25" customHeight="1">
       <c r="A125" s="21"/>
-      <c r="B125" s="79"/>
-      <c r="C125" s="61"/>
+      <c r="B125" s="78"/>
+      <c r="C125" s="60"/>
       <c r="D125" s="41"/>
       <c r="E125" s="41"/>
       <c r="F125" s="40"/>
@@ -6107,38 +5971,38 @@
     </row>
     <row r="126" ht="25.5" customHeight="1">
       <c r="A126" s="21"/>
-      <c r="B126" s="79">
+      <c r="B126" s="78">
         <v>0.9166666666666666</v>
       </c>
       <c r="C126" s="129"/>
       <c r="D126" s="31"/>
       <c r="E126" s="130" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F126" s="131" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G126" s="99" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H126" s="132" t="s">
-        <v>162</v>
-      </c>
-      <c r="I126" s="95" t="s">
         <v>163</v>
       </c>
+      <c r="I126" s="94" t="s">
+        <v>164</v>
+      </c>
       <c r="J126" s="106" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K126" s="126" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L126" s="56" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N126" s="40"/>
       <c r="O126" s="106" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P126" s="40"/>
     </row>
@@ -6146,7 +6010,7 @@
       <c r="A127" s="21"/>
       <c r="B127" s="40"/>
       <c r="C127" s="17"/>
-      <c r="E127" s="66"/>
+      <c r="E127" s="65"/>
       <c r="F127" s="40"/>
       <c r="G127" s="40"/>
       <c r="H127" s="40"/>
@@ -6157,30 +6021,30 @@
     </row>
     <row r="128" ht="54.0" customHeight="1">
       <c r="A128" s="21"/>
-      <c r="B128" s="79">
+      <c r="B128" s="78">
         <v>0.9583333333333334</v>
       </c>
       <c r="C128" s="17"/>
       <c r="D128" s="133" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E128" s="106" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F128" s="40"/>
       <c r="G128" s="100" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H128" s="40"/>
       <c r="I128" s="134" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K128" s="126" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L128" s="40"/>
       <c r="M128" s="135" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N128" s="40"/>
       <c r="P128" s="40"/>
@@ -6188,17 +6052,17 @@
     <row r="129" ht="60.0" customHeight="1">
       <c r="A129" s="21"/>
       <c r="B129" s="41"/>
-      <c r="C129" s="66"/>
+      <c r="C129" s="65"/>
       <c r="D129" s="41"/>
       <c r="F129" s="41"/>
       <c r="G129" s="41"/>
       <c r="H129" s="41"/>
-      <c r="I129" s="95" t="s">
-        <v>163</v>
+      <c r="I129" s="94" t="s">
+        <v>174</v>
       </c>
       <c r="K129" s="41"/>
       <c r="L129" s="41"/>
-      <c r="M129" s="66"/>
+      <c r="M129" s="65"/>
       <c r="N129" s="41"/>
       <c r="P129" s="40"/>
     </row>
@@ -6213,8 +6077,8 @@
       <c r="G130" s="138"/>
       <c r="H130" s="138"/>
       <c r="I130" s="139"/>
-      <c r="J130" s="69"/>
-      <c r="K130" s="88"/>
+      <c r="J130" s="68"/>
+      <c r="K130" s="87"/>
       <c r="L130" s="140"/>
       <c r="M130" s="140"/>
       <c r="N130" s="141"/>
@@ -6223,46 +6087,46 @@
     </row>
     <row r="131" ht="30.0" customHeight="1">
       <c r="A131" s="21"/>
-      <c r="B131" s="79">
+      <c r="B131" s="78">
         <v>1.0</v>
       </c>
       <c r="C131" s="129"/>
       <c r="D131" s="133" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E131" s="106" t="s">
-        <v>168</v>
-      </c>
-      <c r="F131" s="95" t="s">
-        <v>92</v>
+        <v>169</v>
+      </c>
+      <c r="F131" s="94" t="s">
+        <v>90</v>
       </c>
       <c r="G131" s="100" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H131" s="132" t="s">
-        <v>162</v>
-      </c>
-      <c r="I131" s="95" t="s">
-        <v>175</v>
+        <v>177</v>
+      </c>
+      <c r="I131" s="94" t="s">
+        <v>178</v>
       </c>
       <c r="J131" s="106" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K131" s="126" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L131" s="56" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="M131" s="38"/>
-      <c r="N131" s="89" t="s">
-        <v>177</v>
+      <c r="N131" s="88" t="s">
+        <v>180</v>
       </c>
       <c r="O131" s="106" t="s">
-        <v>178</v>
-      </c>
-      <c r="P131" s="127" t="s">
-        <v>179</v>
+        <v>181</v>
+      </c>
+      <c r="P131" s="143" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="132" ht="48.75" customHeight="1">
@@ -6279,18 +6143,18 @@
     </row>
     <row r="133" ht="22.5" customHeight="1">
       <c r="A133" s="21"/>
-      <c r="B133" s="79">
+      <c r="B133" s="78">
         <v>0.041666666666666664</v>
       </c>
       <c r="C133" s="17"/>
       <c r="D133" s="41"/>
       <c r="E133" s="106" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G133" s="40"/>
       <c r="H133" s="41"/>
       <c r="K133" s="100" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="L133" s="41"/>
       <c r="N133" s="40"/>
@@ -6298,7 +6162,7 @@
     </row>
     <row r="134" ht="32.25" customHeight="1">
       <c r="A134" s="21"/>
-      <c r="B134" s="79">
+      <c r="B134" s="78">
         <v>0.08333333333333333</v>
       </c>
       <c r="C134" s="17"/>
@@ -6310,17 +6174,17 @@
       <c r="K134" s="40"/>
       <c r="L134" s="39"/>
       <c r="N134" s="40"/>
-      <c r="O134" s="143"/>
+      <c r="O134" s="144"/>
       <c r="P134" s="40"/>
     </row>
     <row r="135" ht="31.5" customHeight="1">
       <c r="A135" s="21"/>
-      <c r="B135" s="79">
+      <c r="B135" s="78">
         <v>0.125</v>
       </c>
       <c r="C135" s="17"/>
       <c r="E135" s="106" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G135" s="31"/>
       <c r="I135" s="31"/>
@@ -6330,7 +6194,7 @@
     </row>
     <row r="136" ht="27.75" customHeight="1">
       <c r="A136" s="21"/>
-      <c r="B136" s="79">
+      <c r="B136" s="78">
         <v>0.16666666666666666</v>
       </c>
       <c r="C136" s="17"/>
@@ -6340,15 +6204,15 @@
     </row>
     <row r="137" ht="25.5" customHeight="1">
       <c r="A137" s="21"/>
-      <c r="B137" s="79">
+      <c r="B137" s="78">
         <v>0.20833333333333334</v>
       </c>
       <c r="C137" s="17"/>
-      <c r="E137" s="95" t="s">
-        <v>183</v>
+      <c r="E137" s="94" t="s">
+        <v>186</v>
       </c>
       <c r="H137" s="30" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="K137" s="39"/>
       <c r="N137" s="40"/>
@@ -6356,12 +6220,12 @@
     </row>
     <row r="138">
       <c r="A138" s="21"/>
-      <c r="B138" s="77">
+      <c r="B138" s="76">
         <v>0.25</v>
       </c>
       <c r="C138" s="17"/>
       <c r="D138" s="30" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H138" s="40"/>
       <c r="N138" s="41"/>
@@ -6369,13 +6233,13 @@
     </row>
     <row r="139" ht="27.75" customHeight="1">
       <c r="A139" s="21"/>
-      <c r="B139" s="79">
+      <c r="B139" s="78">
         <v>0.2916666666666667</v>
       </c>
       <c r="C139" s="17"/>
       <c r="D139" s="40"/>
-      <c r="E139" s="95" t="s">
-        <v>186</v>
+      <c r="E139" s="94" t="s">
+        <v>189</v>
       </c>
       <c r="H139" s="40"/>
       <c r="N139" s="39"/>
@@ -6383,19 +6247,19 @@
     </row>
     <row r="140" ht="32.25" customHeight="1">
       <c r="A140" s="21"/>
-      <c r="B140" s="79">
+      <c r="B140" s="78">
         <v>0.3333333333333333</v>
       </c>
       <c r="C140" s="17"/>
       <c r="D140" s="40"/>
       <c r="G140" s="37" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H140" s="40"/>
     </row>
     <row r="141" ht="27.75" customHeight="1">
       <c r="A141" s="21"/>
-      <c r="B141" s="79">
+      <c r="B141" s="78">
         <v>0.375</v>
       </c>
       <c r="C141" s="17"/>
@@ -6404,22 +6268,22 @@
       <c r="G141" s="40"/>
       <c r="H141" s="40"/>
       <c r="I141" s="30" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="142" ht="61.5" customHeight="1">
       <c r="A142" s="21"/>
-      <c r="B142" s="79">
+      <c r="B142" s="78">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C142" s="80" t="s">
-        <v>189</v>
+      <c r="C142" s="79" t="s">
+        <v>192</v>
       </c>
       <c r="D142" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="F142" s="64" t="s">
-        <v>40</v>
+        <v>193</v>
+      </c>
+      <c r="F142" s="63" t="s">
+        <v>39</v>
       </c>
       <c r="G142" s="40"/>
       <c r="H142" s="40"/>
@@ -6427,7 +6291,7 @@
     </row>
     <row r="143" ht="61.5" customHeight="1">
       <c r="A143" s="21"/>
-      <c r="B143" s="79"/>
+      <c r="B143" s="78"/>
       <c r="C143" s="40"/>
       <c r="D143" s="41"/>
       <c r="F143" s="38"/>
@@ -6437,15 +6301,15 @@
     </row>
     <row r="144" ht="90.75" customHeight="1">
       <c r="A144" s="21"/>
-      <c r="B144" s="79">
+      <c r="B144" s="78">
         <v>0.4583333333333333</v>
       </c>
       <c r="C144" s="41"/>
       <c r="D144" s="30" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F144" s="56" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G144" s="40"/>
       <c r="H144" s="41"/>
@@ -6453,41 +6317,41 @@
     </row>
     <row r="145" ht="72.0" customHeight="1">
       <c r="A145" s="21"/>
-      <c r="B145" s="79">
+      <c r="B145" s="78">
         <v>0.5</v>
       </c>
-      <c r="C145" s="144" t="s">
-        <v>193</v>
-      </c>
-      <c r="D145" s="64" t="s">
-        <v>194</v>
+      <c r="C145" s="145" t="s">
+        <v>196</v>
+      </c>
+      <c r="D145" s="63" t="s">
+        <v>197</v>
       </c>
       <c r="E145" s="120" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F145" s="40"/>
       <c r="G145" s="40"/>
       <c r="H145" s="31"/>
     </row>
-    <row r="146" ht="60.75" customHeight="1">
+    <row r="146" ht="79.5" customHeight="1">
       <c r="A146" s="21"/>
       <c r="B146" s="97">
         <v>0.5416666666666666</v>
       </c>
-      <c r="C146" s="66"/>
-      <c r="D146" s="83" t="s">
-        <v>196</v>
+      <c r="C146" s="65"/>
+      <c r="D146" s="82" t="s">
+        <v>199</v>
       </c>
       <c r="E146" s="40"/>
       <c r="F146" s="40"/>
       <c r="G146" s="40"/>
     </row>
-    <row r="147" ht="57.75" customHeight="1">
+    <row r="147" ht="69.75" customHeight="1">
       <c r="A147" s="21"/>
       <c r="B147" s="17"/>
-      <c r="C147" s="145"/>
-      <c r="D147" s="83" t="s">
-        <v>197</v>
+      <c r="C147" s="146"/>
+      <c r="D147" s="82" t="s">
+        <v>200</v>
       </c>
       <c r="E147" s="40"/>
       <c r="F147" s="41"/>
@@ -6498,31 +6362,31 @@
       <c r="B148" s="97">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C148" s="146"/>
-      <c r="D148" s="147" t="s">
-        <v>198</v>
+      <c r="C148" s="147"/>
+      <c r="D148" s="148" t="s">
+        <v>201</v>
       </c>
       <c r="E148" s="40"/>
-      <c r="F148" s="148" t="s">
-        <v>199</v>
+      <c r="F148" s="149" t="s">
+        <v>202</v>
       </c>
       <c r="G148" s="38"/>
     </row>
     <row r="149" ht="21.0" customHeight="1">
       <c r="A149" s="21"/>
-      <c r="B149" s="149">
+      <c r="B149" s="150">
         <v>0.625</v>
       </c>
       <c r="C149" s="17"/>
       <c r="D149" s="30" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E149" s="40"/>
       <c r="F149" s="41"/>
     </row>
     <row r="150" ht="36.75" customHeight="1">
       <c r="A150" s="21"/>
-      <c r="B150" s="77">
+      <c r="B150" s="76">
         <v>0.6666666666666666</v>
       </c>
       <c r="C150" s="17"/>
@@ -6539,18 +6403,21 @@
     </row>
     <row r="152" ht="31.5" customHeight="1">
       <c r="A152" s="21"/>
-      <c r="B152" s="79">
+      <c r="B152" s="78">
         <v>0.7083333333333334</v>
       </c>
       <c r="C152" s="17"/>
       <c r="D152" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="E152" s="30" t="s">
-        <v>202</v>
+        <v>204</v>
+      </c>
+      <c r="E152" s="151" t="s">
+        <v>205</v>
+      </c>
+      <c r="F152" s="96" t="s">
+        <v>206</v>
       </c>
       <c r="G152" s="46" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="153" ht="93.75" customHeight="1">
@@ -6559,6 +6426,7 @@
       <c r="C153" s="17"/>
       <c r="D153" s="41"/>
       <c r="E153" s="40"/>
+      <c r="F153" s="41"/>
       <c r="G153" s="40"/>
     </row>
     <row r="154" ht="51.0" customHeight="1">
@@ -6567,16 +6435,16 @@
         <v>0.75</v>
       </c>
       <c r="C154" s="17"/>
-      <c r="D154" s="58" t="s">
-        <v>204</v>
+      <c r="D154" s="96" t="s">
+        <v>208</v>
       </c>
       <c r="E154" s="40"/>
-      <c r="F154" s="64" t="s">
-        <v>62</v>
+      <c r="F154" s="63" t="s">
+        <v>61</v>
       </c>
       <c r="G154" s="41"/>
       <c r="H154" s="56" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="155" ht="34.5" customHeight="1">
@@ -6586,24 +6454,24 @@
       <c r="D155" s="41"/>
       <c r="E155" s="40"/>
       <c r="F155" s="125" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="G155" s="38"/>
       <c r="H155" s="40"/>
     </row>
     <row r="156" ht="77.25" customHeight="1">
       <c r="A156" s="21"/>
-      <c r="B156" s="77">
+      <c r="B156" s="76">
         <v>0.7916666666666666</v>
       </c>
       <c r="C156" s="17"/>
       <c r="D156" s="125" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E156" s="40"/>
       <c r="F156" s="40"/>
       <c r="G156" s="118" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="H156" s="40"/>
     </row>
@@ -6613,27 +6481,27 @@
       <c r="C157" s="17"/>
       <c r="D157" s="41"/>
       <c r="E157" s="41"/>
-      <c r="F157" s="150" t="s">
-        <v>209</v>
+      <c r="F157" s="152" t="s">
+        <v>213</v>
       </c>
       <c r="G157" s="40"/>
       <c r="H157" s="40"/>
     </row>
     <row r="158" ht="75.0" customHeight="1">
       <c r="A158" s="21"/>
-      <c r="B158" s="77">
+      <c r="B158" s="76">
         <v>0.8333333333333334</v>
       </c>
       <c r="C158" s="17"/>
-      <c r="D158" s="151" t="s">
-        <v>210</v>
+      <c r="D158" s="153" t="s">
+        <v>214</v>
       </c>
       <c r="E158" s="56" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F158" s="39"/>
-      <c r="G158" s="152" t="s">
-        <v>212</v>
+      <c r="G158" s="154" t="s">
+        <v>216</v>
       </c>
       <c r="H158" s="40"/>
     </row>
@@ -6641,8 +6509,8 @@
       <c r="A159" s="21"/>
       <c r="B159" s="40"/>
       <c r="C159" s="17"/>
-      <c r="D159" s="58" t="s">
-        <v>213</v>
+      <c r="D159" s="96" t="s">
+        <v>217</v>
       </c>
       <c r="E159" s="40"/>
       <c r="G159" s="40"/>
@@ -6650,7 +6518,7 @@
     </row>
     <row r="160" ht="19.5" customHeight="1">
       <c r="A160" s="21"/>
-      <c r="B160" s="79">
+      <c r="B160" s="78">
         <v>0.875</v>
       </c>
       <c r="C160" s="17"/>
@@ -6661,7 +6529,7 @@
     </row>
     <row r="161" ht="19.5" customHeight="1">
       <c r="A161" s="21"/>
-      <c r="B161" s="77">
+      <c r="B161" s="76">
         <v>0.8958333333333334</v>
       </c>
       <c r="C161" s="17"/>
@@ -6672,7 +6540,7 @@
     </row>
     <row r="162">
       <c r="A162" s="21"/>
-      <c r="B162" s="79">
+      <c r="B162" s="78">
         <v>0.9166666666666666</v>
       </c>
       <c r="C162" s="17"/>
@@ -6683,7 +6551,7 @@
     </row>
     <row r="163">
       <c r="A163" s="21"/>
-      <c r="B163" s="79">
+      <c r="B163" s="78">
         <v>0.9583333333333334</v>
       </c>
       <c r="C163" s="17"/>
@@ -6691,51 +6559,142 @@
     </row>
     <row r="164">
       <c r="A164" s="21"/>
-      <c r="B164" s="79">
+      <c r="B164" s="78">
         <v>1.0</v>
       </c>
       <c r="C164" s="17"/>
       <c r="D164" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="328">
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="B120:B121"/>
-    <mergeCell ref="B107:B108"/>
-    <mergeCell ref="B109:B110"/>
-    <mergeCell ref="C109:C112"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="C113:C121"/>
+  <mergeCells count="329">
+    <mergeCell ref="K94:K106"/>
+    <mergeCell ref="K107:K113"/>
+    <mergeCell ref="M96:M110"/>
+    <mergeCell ref="M111:M114"/>
+    <mergeCell ref="M115:M117"/>
+    <mergeCell ref="H113:H116"/>
+    <mergeCell ref="I113:I115"/>
+    <mergeCell ref="J111:J115"/>
+    <mergeCell ref="J116:J117"/>
+    <mergeCell ref="H85:H88"/>
+    <mergeCell ref="H90:H102"/>
+    <mergeCell ref="L94:L104"/>
+    <mergeCell ref="H103:H104"/>
+    <mergeCell ref="H105:H108"/>
+    <mergeCell ref="L105:L117"/>
+    <mergeCell ref="K114:K117"/>
+    <mergeCell ref="J94:J100"/>
+    <mergeCell ref="J101:J110"/>
+    <mergeCell ref="J118:J121"/>
+    <mergeCell ref="K118:K121"/>
+    <mergeCell ref="L118:L121"/>
+    <mergeCell ref="M118:M121"/>
+    <mergeCell ref="J122:J123"/>
+    <mergeCell ref="M122:M123"/>
+    <mergeCell ref="N131:N138"/>
+    <mergeCell ref="O134:O164"/>
+    <mergeCell ref="N139:N164"/>
+    <mergeCell ref="P139:P164"/>
+    <mergeCell ref="J134:J164"/>
+    <mergeCell ref="I144:I164"/>
+    <mergeCell ref="K122:K125"/>
+    <mergeCell ref="L122:L125"/>
+    <mergeCell ref="J124:J125"/>
+    <mergeCell ref="M131:M164"/>
+    <mergeCell ref="K133:K136"/>
+    <mergeCell ref="L134:L164"/>
+    <mergeCell ref="K137:K164"/>
+    <mergeCell ref="G126:G127"/>
+    <mergeCell ref="G128:G129"/>
+    <mergeCell ref="G94:G104"/>
+    <mergeCell ref="G105:G108"/>
+    <mergeCell ref="G110:G111"/>
+    <mergeCell ref="G113:G115"/>
+    <mergeCell ref="G116:G119"/>
+    <mergeCell ref="G120:G122"/>
+    <mergeCell ref="G123:G124"/>
+    <mergeCell ref="H134:H136"/>
+    <mergeCell ref="H137:H144"/>
+    <mergeCell ref="H145:H153"/>
+    <mergeCell ref="H154:H161"/>
+    <mergeCell ref="H162:H164"/>
+    <mergeCell ref="G140:G147"/>
+    <mergeCell ref="G148:G151"/>
+    <mergeCell ref="G152:G154"/>
+    <mergeCell ref="G156:G157"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="G162:G164"/>
+    <mergeCell ref="H109:H110"/>
+    <mergeCell ref="H111:H112"/>
+    <mergeCell ref="H118:H119"/>
+    <mergeCell ref="H120:H121"/>
+    <mergeCell ref="H122:H124"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="G135:G139"/>
+    <mergeCell ref="G79:G82"/>
+    <mergeCell ref="H79:H82"/>
+    <mergeCell ref="I81:I82"/>
+    <mergeCell ref="G83:G88"/>
+    <mergeCell ref="H83:H84"/>
+    <mergeCell ref="I84:I88"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="I90:I93"/>
+    <mergeCell ref="J81:J84"/>
+    <mergeCell ref="J85:J88"/>
+    <mergeCell ref="J90:J93"/>
+    <mergeCell ref="K90:K93"/>
+    <mergeCell ref="L90:L93"/>
+    <mergeCell ref="M90:M94"/>
+    <mergeCell ref="N90:N94"/>
+    <mergeCell ref="N116:N119"/>
+    <mergeCell ref="N120:N121"/>
+    <mergeCell ref="M124:M127"/>
+    <mergeCell ref="N122:N123"/>
+    <mergeCell ref="N124:N129"/>
+    <mergeCell ref="J126:J129"/>
+    <mergeCell ref="K126:K127"/>
+    <mergeCell ref="L126:L129"/>
+    <mergeCell ref="K128:K129"/>
+    <mergeCell ref="M128:M129"/>
+    <mergeCell ref="O126:O129"/>
+    <mergeCell ref="O131:O133"/>
+    <mergeCell ref="P131:P138"/>
+    <mergeCell ref="O90:O93"/>
+    <mergeCell ref="P90:P100"/>
+    <mergeCell ref="O94:O100"/>
+    <mergeCell ref="N96:N115"/>
+    <mergeCell ref="O101:O125"/>
+    <mergeCell ref="P101:P117"/>
+    <mergeCell ref="P118:P129"/>
+    <mergeCell ref="I135:I140"/>
+    <mergeCell ref="I141:I143"/>
+    <mergeCell ref="I94:I104"/>
+    <mergeCell ref="I105:I112"/>
+    <mergeCell ref="I116:I119"/>
+    <mergeCell ref="I120:I121"/>
+    <mergeCell ref="I122:I123"/>
+    <mergeCell ref="I124:I125"/>
+    <mergeCell ref="I126:I127"/>
     <mergeCell ref="B114:B115"/>
     <mergeCell ref="B116:B117"/>
+    <mergeCell ref="C131:C141"/>
     <mergeCell ref="D131:D133"/>
     <mergeCell ref="D134:D137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="B156:B157"/>
+    <mergeCell ref="D156:D157"/>
+    <mergeCell ref="B158:B159"/>
+    <mergeCell ref="D159:D160"/>
+    <mergeCell ref="D161:D164"/>
+    <mergeCell ref="C142:C144"/>
+    <mergeCell ref="C145:C146"/>
+    <mergeCell ref="B146:B147"/>
+    <mergeCell ref="C148:C164"/>
     <mergeCell ref="D149:D151"/>
     <mergeCell ref="D152:D153"/>
     <mergeCell ref="D154:D155"/>
-    <mergeCell ref="D156:D157"/>
-    <mergeCell ref="D159:D160"/>
-    <mergeCell ref="D161:D164"/>
-    <mergeCell ref="C131:C141"/>
-    <mergeCell ref="C142:C144"/>
-    <mergeCell ref="C145:C146"/>
-    <mergeCell ref="C148:C164"/>
-    <mergeCell ref="B131:B132"/>
-    <mergeCell ref="B146:B147"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="B152:B153"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="B156:B157"/>
-    <mergeCell ref="B158:B159"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="D126:D127"/>
-    <mergeCell ref="B128:B129"/>
-    <mergeCell ref="D128:D129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="D53:D54"/>
     <mergeCell ref="D45:D46"/>
     <mergeCell ref="B47:B48"/>
     <mergeCell ref="C47:C51"/>
@@ -6743,6 +6702,7 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="B53:B54"/>
+    <mergeCell ref="D51:D52"/>
     <mergeCell ref="B66:B67"/>
     <mergeCell ref="B69:B70"/>
     <mergeCell ref="B71:B72"/>
@@ -6750,154 +6710,20 @@
     <mergeCell ref="D75:D76"/>
     <mergeCell ref="B77:B78"/>
     <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D103:D104"/>
-    <mergeCell ref="D105:D106"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="D91:D94"/>
+    <mergeCell ref="B103:B104"/>
+    <mergeCell ref="B105:B106"/>
     <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C81:C83"/>
     <mergeCell ref="B83:B84"/>
     <mergeCell ref="B85:B86"/>
     <mergeCell ref="B87:B88"/>
     <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B103:B104"/>
-    <mergeCell ref="B105:B106"/>
-    <mergeCell ref="D107:D108"/>
-    <mergeCell ref="D109:D110"/>
-    <mergeCell ref="D111:D112"/>
-    <mergeCell ref="D114:D115"/>
-    <mergeCell ref="D116:D117"/>
-    <mergeCell ref="D118:D119"/>
-    <mergeCell ref="D91:D94"/>
-    <mergeCell ref="D95:D101"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D79:D82"/>
-    <mergeCell ref="C89:D89"/>
     <mergeCell ref="C90:C107"/>
-    <mergeCell ref="D87:D88"/>
-    <mergeCell ref="D85:D86"/>
-    <mergeCell ref="L94:L104"/>
-    <mergeCell ref="L105:L117"/>
-    <mergeCell ref="J101:J110"/>
-    <mergeCell ref="J111:J115"/>
-    <mergeCell ref="I105:I112"/>
-    <mergeCell ref="I113:I115"/>
-    <mergeCell ref="M111:M114"/>
-    <mergeCell ref="M115:M117"/>
-    <mergeCell ref="I90:I93"/>
-    <mergeCell ref="I94:I104"/>
-    <mergeCell ref="J94:J100"/>
-    <mergeCell ref="K94:K106"/>
-    <mergeCell ref="M96:M110"/>
-    <mergeCell ref="K107:K113"/>
-    <mergeCell ref="K114:K117"/>
-    <mergeCell ref="J116:J117"/>
-    <mergeCell ref="O101:O125"/>
-    <mergeCell ref="O126:O129"/>
-    <mergeCell ref="M131:M164"/>
-    <mergeCell ref="N131:N138"/>
-    <mergeCell ref="O131:O133"/>
-    <mergeCell ref="O134:O164"/>
-    <mergeCell ref="N139:N164"/>
-    <mergeCell ref="P139:P164"/>
-    <mergeCell ref="N96:N115"/>
-    <mergeCell ref="P101:P117"/>
-    <mergeCell ref="N116:N119"/>
-    <mergeCell ref="P118:P129"/>
-    <mergeCell ref="N120:N121"/>
-    <mergeCell ref="N122:N123"/>
-    <mergeCell ref="N124:N129"/>
-    <mergeCell ref="P131:P138"/>
-    <mergeCell ref="J126:J129"/>
-    <mergeCell ref="I130:K130"/>
-    <mergeCell ref="E126:E127"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="G126:G127"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="I126:I127"/>
-    <mergeCell ref="E128:E129"/>
-    <mergeCell ref="G128:G129"/>
-    <mergeCell ref="J81:J84"/>
-    <mergeCell ref="J85:J88"/>
-    <mergeCell ref="J90:J93"/>
-    <mergeCell ref="K90:K93"/>
-    <mergeCell ref="L90:L93"/>
-    <mergeCell ref="M90:M94"/>
-    <mergeCell ref="N90:N94"/>
-    <mergeCell ref="O90:O93"/>
-    <mergeCell ref="G79:G82"/>
-    <mergeCell ref="H79:H82"/>
-    <mergeCell ref="I81:I82"/>
-    <mergeCell ref="G83:G88"/>
-    <mergeCell ref="H83:H84"/>
-    <mergeCell ref="I84:I88"/>
-    <mergeCell ref="H85:H88"/>
-    <mergeCell ref="K118:K121"/>
-    <mergeCell ref="K122:K125"/>
-    <mergeCell ref="L122:L125"/>
-    <mergeCell ref="M124:M127"/>
-    <mergeCell ref="K126:K127"/>
-    <mergeCell ref="L126:L129"/>
-    <mergeCell ref="K128:K129"/>
-    <mergeCell ref="M128:M129"/>
-    <mergeCell ref="F122:F123"/>
-    <mergeCell ref="F124:F125"/>
-    <mergeCell ref="I124:I125"/>
-    <mergeCell ref="J124:J125"/>
-    <mergeCell ref="F94:F102"/>
-    <mergeCell ref="F103:F104"/>
-    <mergeCell ref="F105:F106"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="F107:F113"/>
-    <mergeCell ref="E109:E113"/>
-    <mergeCell ref="F114:F121"/>
-    <mergeCell ref="E96:E102"/>
-    <mergeCell ref="E131:E132"/>
-    <mergeCell ref="E133:E134"/>
-    <mergeCell ref="F134:F141"/>
-    <mergeCell ref="E135:E136"/>
-    <mergeCell ref="E137:E138"/>
-    <mergeCell ref="E139:E140"/>
-    <mergeCell ref="E141:E144"/>
-    <mergeCell ref="F81:F84"/>
-    <mergeCell ref="F85:F88"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E90:E95"/>
-    <mergeCell ref="E83:E87"/>
-    <mergeCell ref="H90:H102"/>
-    <mergeCell ref="E80:E82"/>
-    <mergeCell ref="F131:F133"/>
-    <mergeCell ref="G131:G134"/>
-    <mergeCell ref="I131:I134"/>
-    <mergeCell ref="J131:J133"/>
-    <mergeCell ref="K131:K132"/>
-    <mergeCell ref="L131:L133"/>
-    <mergeCell ref="K133:K136"/>
-    <mergeCell ref="G135:G139"/>
-    <mergeCell ref="G158:G161"/>
-    <mergeCell ref="G162:G164"/>
-    <mergeCell ref="H131:H133"/>
-    <mergeCell ref="H134:H136"/>
-    <mergeCell ref="L134:L164"/>
-    <mergeCell ref="K137:K164"/>
-    <mergeCell ref="F144:F147"/>
-    <mergeCell ref="F148:F149"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="H162:H164"/>
-    <mergeCell ref="I135:I140"/>
-    <mergeCell ref="I141:I143"/>
-    <mergeCell ref="J134:J164"/>
-    <mergeCell ref="I144:I164"/>
-    <mergeCell ref="H137:H144"/>
-    <mergeCell ref="H145:H153"/>
-    <mergeCell ref="G140:G147"/>
-    <mergeCell ref="G148:G151"/>
-    <mergeCell ref="E145:E151"/>
-    <mergeCell ref="E152:E157"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="E162:E164"/>
-    <mergeCell ref="G152:G154"/>
-    <mergeCell ref="H154:H161"/>
-    <mergeCell ref="G156:G157"/>
-    <mergeCell ref="F155:F156"/>
-    <mergeCell ref="F158:F164"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="B154:B155"/>
+    <mergeCell ref="D53:D54"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="D11:D14"/>
     <mergeCell ref="E11:E14"/>
@@ -6949,8 +6775,6 @@
     <mergeCell ref="M79:M82"/>
     <mergeCell ref="N75:N86"/>
     <mergeCell ref="O81:O84"/>
-    <mergeCell ref="P90:P100"/>
-    <mergeCell ref="O94:O100"/>
     <mergeCell ref="L78:L84"/>
     <mergeCell ref="L85:L88"/>
     <mergeCell ref="M83:M86"/>
@@ -6967,6 +6791,8 @@
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="E60:E61"/>
     <mergeCell ref="E73:E79"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="E83:E87"/>
     <mergeCell ref="D26:D29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D31:D34"/>
@@ -6979,7 +6805,6 @@
     <mergeCell ref="C61:C64"/>
     <mergeCell ref="C66:C68"/>
     <mergeCell ref="C69:C80"/>
-    <mergeCell ref="C81:C83"/>
     <mergeCell ref="C85:C88"/>
     <mergeCell ref="D56:D58"/>
     <mergeCell ref="D69:D72"/>
@@ -6994,39 +6819,83 @@
     <mergeCell ref="H75:H78"/>
     <mergeCell ref="F76:F78"/>
     <mergeCell ref="F79:F80"/>
-    <mergeCell ref="G90:G93"/>
-    <mergeCell ref="G94:G104"/>
-    <mergeCell ref="G105:G108"/>
-    <mergeCell ref="G110:G111"/>
-    <mergeCell ref="G113:G115"/>
-    <mergeCell ref="G116:G119"/>
-    <mergeCell ref="H103:H104"/>
-    <mergeCell ref="H105:H108"/>
-    <mergeCell ref="H109:H110"/>
-    <mergeCell ref="H111:H112"/>
-    <mergeCell ref="H113:H116"/>
-    <mergeCell ref="I116:I119"/>
-    <mergeCell ref="H118:H119"/>
-    <mergeCell ref="I120:I121"/>
-    <mergeCell ref="I122:I123"/>
-    <mergeCell ref="G120:G122"/>
-    <mergeCell ref="G123:G124"/>
-    <mergeCell ref="J118:J121"/>
-    <mergeCell ref="L118:L121"/>
-    <mergeCell ref="M118:M121"/>
-    <mergeCell ref="H120:H121"/>
-    <mergeCell ref="H122:H124"/>
-    <mergeCell ref="J122:J123"/>
-    <mergeCell ref="M122:M123"/>
+    <mergeCell ref="F81:F84"/>
+    <mergeCell ref="F85:F88"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="F94:F102"/>
+    <mergeCell ref="E96:E102"/>
+    <mergeCell ref="F103:F104"/>
+    <mergeCell ref="F105:F106"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="F107:F113"/>
+    <mergeCell ref="E109:E113"/>
+    <mergeCell ref="E114:E116"/>
+    <mergeCell ref="F114:F121"/>
+    <mergeCell ref="E118:E119"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="F122:F123"/>
+    <mergeCell ref="E124:E125"/>
+    <mergeCell ref="F124:F125"/>
+    <mergeCell ref="E126:E127"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E128:E129"/>
+    <mergeCell ref="F144:F147"/>
+    <mergeCell ref="F148:F149"/>
+    <mergeCell ref="F158:F164"/>
+    <mergeCell ref="F152:F153"/>
+    <mergeCell ref="F150:F151"/>
+    <mergeCell ref="E145:E151"/>
+    <mergeCell ref="E152:E157"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="E162:E164"/>
+    <mergeCell ref="F131:F133"/>
+    <mergeCell ref="F134:F141"/>
+    <mergeCell ref="E135:E136"/>
+    <mergeCell ref="E137:E138"/>
+    <mergeCell ref="E139:E140"/>
+    <mergeCell ref="E141:E144"/>
+    <mergeCell ref="F155:F156"/>
+    <mergeCell ref="D107:D108"/>
+    <mergeCell ref="D109:D110"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D79:D82"/>
+    <mergeCell ref="D85:D86"/>
+    <mergeCell ref="D87:D88"/>
+    <mergeCell ref="D95:D101"/>
+    <mergeCell ref="D103:D104"/>
+    <mergeCell ref="D105:D106"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="C113:C121"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="B107:B108"/>
+    <mergeCell ref="B109:B110"/>
+    <mergeCell ref="C109:C112"/>
+    <mergeCell ref="D111:D112"/>
+    <mergeCell ref="D114:D115"/>
+    <mergeCell ref="D116:D117"/>
+    <mergeCell ref="D118:D119"/>
+    <mergeCell ref="D126:D127"/>
+    <mergeCell ref="D128:D129"/>
+    <mergeCell ref="I130:K130"/>
+    <mergeCell ref="D120:D123"/>
     <mergeCell ref="B122:B123"/>
+    <mergeCell ref="C122:C124"/>
+    <mergeCell ref="D124:D125"/>
     <mergeCell ref="B126:B127"/>
-    <mergeCell ref="E114:E116"/>
-    <mergeCell ref="E118:E119"/>
-    <mergeCell ref="D120:D123"/>
-    <mergeCell ref="C122:C124"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="D124:D125"/>
-    <mergeCell ref="E124:E125"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="K131:K132"/>
+    <mergeCell ref="L131:L133"/>
+    <mergeCell ref="B128:B129"/>
+    <mergeCell ref="B131:B132"/>
+    <mergeCell ref="E131:E132"/>
+    <mergeCell ref="G131:G134"/>
+    <mergeCell ref="H131:H133"/>
+    <mergeCell ref="I131:I134"/>
+    <mergeCell ref="J131:J133"/>
+    <mergeCell ref="E133:E134"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId4" ref="F148"/>
@@ -7054,394 +6923,394 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="153" t="s">
-        <v>214</v>
-      </c>
-      <c r="C1" s="153" t="s">
-        <v>215</v>
-      </c>
-      <c r="D1" s="153" t="s">
-        <v>216</v>
-      </c>
-      <c r="E1" s="153" t="s">
-        <v>217</v>
+      <c r="B1" s="155" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" s="155" t="s">
+        <v>219</v>
+      </c>
+      <c r="D1" s="155" t="s">
+        <v>220</v>
+      </c>
+      <c r="E1" s="155" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="154" t="s">
-        <v>218</v>
-      </c>
-      <c r="B2" s="155"/>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="155"/>
-      <c r="L2" s="155"/>
-      <c r="M2" s="155"/>
-      <c r="N2" s="155"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="155"/>
-      <c r="Q2" s="155"/>
-      <c r="R2" s="155"/>
-      <c r="S2" s="155"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="155"/>
-      <c r="V2" s="155"/>
-      <c r="W2" s="155"/>
-      <c r="X2" s="155"/>
-      <c r="Y2" s="155"/>
-      <c r="Z2" s="155"/>
-      <c r="AA2" s="156"/>
+      <c r="A2" s="156" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="157"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="157"/>
+      <c r="P2" s="157"/>
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="157"/>
+      <c r="U2" s="157"/>
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="158"/>
     </row>
     <row r="3">
-      <c r="A3" s="157"/>
-      <c r="B3" s="153" t="s">
-        <v>219</v>
-      </c>
-      <c r="E3" s="153" t="s">
-        <v>220</v>
-      </c>
-      <c r="AA3" s="158"/>
+      <c r="A3" s="159"/>
+      <c r="B3" s="155" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="155" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA3" s="160"/>
     </row>
     <row r="4">
-      <c r="A4" s="157"/>
-      <c r="B4" s="153" t="s">
-        <v>221</v>
-      </c>
-      <c r="E4" s="153" t="s">
-        <v>222</v>
-      </c>
-      <c r="AA4" s="158"/>
+      <c r="A4" s="159"/>
+      <c r="B4" s="155" t="s">
+        <v>225</v>
+      </c>
+      <c r="E4" s="155" t="s">
+        <v>226</v>
+      </c>
+      <c r="AA4" s="160"/>
     </row>
     <row r="5">
-      <c r="A5" s="159"/>
-      <c r="B5" s="160" t="s">
-        <v>223</v>
-      </c>
-      <c r="C5" s="161"/>
-      <c r="D5" s="161"/>
-      <c r="E5" s="160" t="s">
-        <v>224</v>
-      </c>
-      <c r="F5" s="161"/>
-      <c r="G5" s="161"/>
-      <c r="H5" s="161"/>
-      <c r="I5" s="161"/>
-      <c r="J5" s="161"/>
-      <c r="K5" s="161"/>
-      <c r="L5" s="161"/>
-      <c r="M5" s="161"/>
-      <c r="N5" s="161"/>
-      <c r="O5" s="161"/>
-      <c r="P5" s="161"/>
-      <c r="Q5" s="161"/>
-      <c r="R5" s="161"/>
-      <c r="S5" s="161"/>
-      <c r="T5" s="161"/>
-      <c r="U5" s="161"/>
-      <c r="V5" s="161"/>
-      <c r="W5" s="161"/>
-      <c r="X5" s="161"/>
-      <c r="Y5" s="161"/>
-      <c r="Z5" s="161"/>
-      <c r="AA5" s="162"/>
+      <c r="A5" s="161"/>
+      <c r="B5" s="162" t="s">
+        <v>227</v>
+      </c>
+      <c r="C5" s="163"/>
+      <c r="D5" s="163"/>
+      <c r="E5" s="162" t="s">
+        <v>228</v>
+      </c>
+      <c r="F5" s="163"/>
+      <c r="G5" s="163"/>
+      <c r="H5" s="163"/>
+      <c r="I5" s="163"/>
+      <c r="J5" s="163"/>
+      <c r="K5" s="163"/>
+      <c r="L5" s="163"/>
+      <c r="M5" s="163"/>
+      <c r="N5" s="163"/>
+      <c r="O5" s="163"/>
+      <c r="P5" s="163"/>
+      <c r="Q5" s="163"/>
+      <c r="R5" s="163"/>
+      <c r="S5" s="163"/>
+      <c r="T5" s="163"/>
+      <c r="U5" s="163"/>
+      <c r="V5" s="163"/>
+      <c r="W5" s="163"/>
+      <c r="X5" s="163"/>
+      <c r="Y5" s="163"/>
+      <c r="Z5" s="163"/>
+      <c r="AA5" s="164"/>
     </row>
     <row r="6">
-      <c r="A6" s="154" t="s">
-        <v>225</v>
-      </c>
-      <c r="B6" s="163"/>
-      <c r="C6" s="155"/>
-      <c r="D6" s="155"/>
-      <c r="E6" s="155"/>
-      <c r="F6" s="155"/>
-      <c r="G6" s="155"/>
-      <c r="H6" s="155"/>
-      <c r="I6" s="155"/>
-      <c r="J6" s="155"/>
-      <c r="K6" s="155"/>
-      <c r="L6" s="155"/>
-      <c r="M6" s="155"/>
-      <c r="N6" s="155"/>
-      <c r="O6" s="155"/>
-      <c r="P6" s="155"/>
-      <c r="Q6" s="155"/>
-      <c r="R6" s="155"/>
-      <c r="S6" s="155"/>
-      <c r="T6" s="155"/>
-      <c r="U6" s="155"/>
-      <c r="V6" s="155"/>
-      <c r="W6" s="155"/>
-      <c r="X6" s="155"/>
-      <c r="Y6" s="155"/>
-      <c r="Z6" s="155"/>
-      <c r="AA6" s="156"/>
+      <c r="A6" s="156" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="165"/>
+      <c r="C6" s="157"/>
+      <c r="D6" s="157"/>
+      <c r="E6" s="157"/>
+      <c r="F6" s="157"/>
+      <c r="G6" s="157"/>
+      <c r="H6" s="157"/>
+      <c r="I6" s="157"/>
+      <c r="J6" s="157"/>
+      <c r="K6" s="157"/>
+      <c r="L6" s="157"/>
+      <c r="M6" s="157"/>
+      <c r="N6" s="157"/>
+      <c r="O6" s="157"/>
+      <c r="P6" s="157"/>
+      <c r="Q6" s="157"/>
+      <c r="R6" s="157"/>
+      <c r="S6" s="157"/>
+      <c r="T6" s="157"/>
+      <c r="U6" s="157"/>
+      <c r="V6" s="157"/>
+      <c r="W6" s="157"/>
+      <c r="X6" s="157"/>
+      <c r="Y6" s="157"/>
+      <c r="Z6" s="157"/>
+      <c r="AA6" s="158"/>
     </row>
     <row r="7">
-      <c r="A7" s="157"/>
-      <c r="B7" s="153" t="s">
-        <v>226</v>
-      </c>
-      <c r="E7" s="153" t="s">
-        <v>227</v>
-      </c>
-      <c r="AA7" s="158"/>
+      <c r="A7" s="159"/>
+      <c r="B7" s="155" t="s">
+        <v>230</v>
+      </c>
+      <c r="E7" s="155" t="s">
+        <v>231</v>
+      </c>
+      <c r="AA7" s="160"/>
     </row>
     <row r="8">
-      <c r="A8" s="157"/>
-      <c r="B8" s="153" t="s">
-        <v>228</v>
-      </c>
-      <c r="E8" s="153" t="s">
-        <v>229</v>
-      </c>
-      <c r="AA8" s="158"/>
+      <c r="A8" s="159"/>
+      <c r="B8" s="155" t="s">
+        <v>232</v>
+      </c>
+      <c r="E8" s="155" t="s">
+        <v>233</v>
+      </c>
+      <c r="AA8" s="160"/>
     </row>
     <row r="9">
-      <c r="A9" s="157"/>
-      <c r="B9" s="153" t="s">
-        <v>230</v>
-      </c>
-      <c r="E9" s="153" t="s">
-        <v>231</v>
-      </c>
-      <c r="AA9" s="158"/>
+      <c r="A9" s="159"/>
+      <c r="B9" s="155" t="s">
+        <v>234</v>
+      </c>
+      <c r="E9" s="155" t="s">
+        <v>235</v>
+      </c>
+      <c r="AA9" s="160"/>
     </row>
     <row r="10">
-      <c r="A10" s="157"/>
-      <c r="B10" s="153" t="s">
-        <v>232</v>
-      </c>
-      <c r="E10" s="153" t="s">
-        <v>233</v>
-      </c>
-      <c r="AA10" s="158"/>
+      <c r="A10" s="159"/>
+      <c r="B10" s="155" t="s">
+        <v>236</v>
+      </c>
+      <c r="E10" s="155" t="s">
+        <v>237</v>
+      </c>
+      <c r="AA10" s="160"/>
     </row>
     <row r="11">
-      <c r="A11" s="159"/>
-      <c r="B11" s="160" t="s">
-        <v>234</v>
-      </c>
-      <c r="D11" s="161"/>
-      <c r="E11" s="160" t="s">
-        <v>235</v>
-      </c>
-      <c r="F11" s="161"/>
-      <c r="G11" s="161"/>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="161"/>
-      <c r="K11" s="161"/>
-      <c r="L11" s="161"/>
-      <c r="M11" s="161"/>
-      <c r="N11" s="161"/>
-      <c r="O11" s="161"/>
-      <c r="P11" s="161"/>
-      <c r="Q11" s="161"/>
-      <c r="R11" s="161"/>
-      <c r="S11" s="161"/>
-      <c r="T11" s="161"/>
-      <c r="U11" s="161"/>
-      <c r="V11" s="161"/>
-      <c r="W11" s="161"/>
-      <c r="X11" s="161"/>
-      <c r="Y11" s="161"/>
-      <c r="Z11" s="161"/>
-      <c r="AA11" s="162"/>
+      <c r="A11" s="161"/>
+      <c r="B11" s="162" t="s">
+        <v>238</v>
+      </c>
+      <c r="D11" s="163"/>
+      <c r="E11" s="162" t="s">
+        <v>239</v>
+      </c>
+      <c r="F11" s="163"/>
+      <c r="G11" s="163"/>
+      <c r="H11" s="163"/>
+      <c r="I11" s="163"/>
+      <c r="J11" s="163"/>
+      <c r="K11" s="163"/>
+      <c r="L11" s="163"/>
+      <c r="M11" s="163"/>
+      <c r="N11" s="163"/>
+      <c r="O11" s="163"/>
+      <c r="P11" s="163"/>
+      <c r="Q11" s="163"/>
+      <c r="R11" s="163"/>
+      <c r="S11" s="163"/>
+      <c r="T11" s="163"/>
+      <c r="U11" s="163"/>
+      <c r="V11" s="163"/>
+      <c r="W11" s="163"/>
+      <c r="X11" s="163"/>
+      <c r="Y11" s="163"/>
+      <c r="Z11" s="163"/>
+      <c r="AA11" s="164"/>
     </row>
     <row r="12">
-      <c r="A12" s="154" t="s">
-        <v>236</v>
-      </c>
-      <c r="B12" s="155"/>
-      <c r="C12" s="155"/>
-      <c r="D12" s="155"/>
-      <c r="E12" s="155"/>
-      <c r="F12" s="155"/>
-      <c r="G12" s="155"/>
-      <c r="H12" s="155"/>
-      <c r="I12" s="155"/>
-      <c r="J12" s="155"/>
-      <c r="K12" s="155"/>
-      <c r="L12" s="155"/>
-      <c r="M12" s="155"/>
-      <c r="N12" s="155"/>
-      <c r="O12" s="155"/>
-      <c r="P12" s="155"/>
-      <c r="Q12" s="155"/>
-      <c r="R12" s="155"/>
-      <c r="S12" s="155"/>
-      <c r="T12" s="155"/>
-      <c r="U12" s="155"/>
-      <c r="V12" s="155"/>
-      <c r="W12" s="155"/>
-      <c r="X12" s="155"/>
-      <c r="Y12" s="155"/>
-      <c r="Z12" s="155"/>
-      <c r="AA12" s="156"/>
+      <c r="A12" s="156" t="s">
+        <v>240</v>
+      </c>
+      <c r="B12" s="157"/>
+      <c r="C12" s="157"/>
+      <c r="D12" s="157"/>
+      <c r="E12" s="157"/>
+      <c r="F12" s="157"/>
+      <c r="G12" s="157"/>
+      <c r="H12" s="157"/>
+      <c r="I12" s="157"/>
+      <c r="J12" s="157"/>
+      <c r="K12" s="157"/>
+      <c r="L12" s="157"/>
+      <c r="M12" s="157"/>
+      <c r="N12" s="157"/>
+      <c r="O12" s="157"/>
+      <c r="P12" s="157"/>
+      <c r="Q12" s="157"/>
+      <c r="R12" s="157"/>
+      <c r="S12" s="157"/>
+      <c r="T12" s="157"/>
+      <c r="U12" s="157"/>
+      <c r="V12" s="157"/>
+      <c r="W12" s="157"/>
+      <c r="X12" s="157"/>
+      <c r="Y12" s="157"/>
+      <c r="Z12" s="157"/>
+      <c r="AA12" s="158"/>
     </row>
     <row r="13">
-      <c r="A13" s="157"/>
-      <c r="B13" s="153" t="s">
-        <v>237</v>
-      </c>
-      <c r="E13" s="153" t="s">
-        <v>238</v>
-      </c>
-      <c r="AA13" s="158"/>
+      <c r="A13" s="159"/>
+      <c r="B13" s="155" t="s">
+        <v>241</v>
+      </c>
+      <c r="E13" s="155" t="s">
+        <v>242</v>
+      </c>
+      <c r="AA13" s="160"/>
     </row>
     <row r="14">
-      <c r="A14" s="159"/>
-      <c r="B14" s="160" t="s">
-        <v>239</v>
-      </c>
-      <c r="C14" s="161"/>
-      <c r="D14" s="161"/>
-      <c r="E14" s="160" t="s">
-        <v>240</v>
-      </c>
-      <c r="F14" s="161"/>
-      <c r="G14" s="161"/>
-      <c r="H14" s="161"/>
-      <c r="I14" s="161"/>
-      <c r="J14" s="161"/>
-      <c r="K14" s="161"/>
-      <c r="L14" s="161"/>
-      <c r="M14" s="161"/>
-      <c r="N14" s="161"/>
-      <c r="O14" s="161"/>
-      <c r="P14" s="161"/>
-      <c r="Q14" s="161"/>
-      <c r="R14" s="161"/>
-      <c r="S14" s="161"/>
-      <c r="T14" s="161"/>
-      <c r="U14" s="161"/>
-      <c r="V14" s="161"/>
-      <c r="W14" s="161"/>
-      <c r="X14" s="161"/>
-      <c r="Y14" s="161"/>
-      <c r="Z14" s="161"/>
-      <c r="AA14" s="162"/>
+      <c r="A14" s="161"/>
+      <c r="B14" s="162" t="s">
+        <v>243</v>
+      </c>
+      <c r="C14" s="163"/>
+      <c r="D14" s="163"/>
+      <c r="E14" s="162" t="s">
+        <v>244</v>
+      </c>
+      <c r="F14" s="163"/>
+      <c r="G14" s="163"/>
+      <c r="H14" s="163"/>
+      <c r="I14" s="163"/>
+      <c r="J14" s="163"/>
+      <c r="K14" s="163"/>
+      <c r="L14" s="163"/>
+      <c r="M14" s="163"/>
+      <c r="N14" s="163"/>
+      <c r="O14" s="163"/>
+      <c r="P14" s="163"/>
+      <c r="Q14" s="163"/>
+      <c r="R14" s="163"/>
+      <c r="S14" s="163"/>
+      <c r="T14" s="163"/>
+      <c r="U14" s="163"/>
+      <c r="V14" s="163"/>
+      <c r="W14" s="163"/>
+      <c r="X14" s="163"/>
+      <c r="Y14" s="163"/>
+      <c r="Z14" s="163"/>
+      <c r="AA14" s="164"/>
     </row>
     <row r="15">
-      <c r="A15" s="154" t="s">
-        <v>241</v>
-      </c>
-      <c r="B15" s="155"/>
-      <c r="C15" s="155"/>
-      <c r="D15" s="155"/>
-      <c r="E15" s="155"/>
-      <c r="F15" s="155"/>
-      <c r="G15" s="155"/>
-      <c r="H15" s="155"/>
-      <c r="I15" s="155"/>
-      <c r="J15" s="155"/>
-      <c r="K15" s="155"/>
-      <c r="L15" s="155"/>
-      <c r="M15" s="155"/>
-      <c r="N15" s="155"/>
-      <c r="O15" s="155"/>
-      <c r="P15" s="155"/>
-      <c r="Q15" s="155"/>
-      <c r="R15" s="155"/>
-      <c r="S15" s="155"/>
-      <c r="T15" s="155"/>
-      <c r="U15" s="155"/>
-      <c r="V15" s="155"/>
-      <c r="W15" s="155"/>
-      <c r="X15" s="155"/>
-      <c r="Y15" s="155"/>
-      <c r="Z15" s="155"/>
-      <c r="AA15" s="156"/>
+      <c r="A15" s="156" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" s="157"/>
+      <c r="C15" s="157"/>
+      <c r="D15" s="157"/>
+      <c r="E15" s="157"/>
+      <c r="F15" s="157"/>
+      <c r="G15" s="157"/>
+      <c r="H15" s="157"/>
+      <c r="I15" s="157"/>
+      <c r="J15" s="157"/>
+      <c r="K15" s="157"/>
+      <c r="L15" s="157"/>
+      <c r="M15" s="157"/>
+      <c r="N15" s="157"/>
+      <c r="O15" s="157"/>
+      <c r="P15" s="157"/>
+      <c r="Q15" s="157"/>
+      <c r="R15" s="157"/>
+      <c r="S15" s="157"/>
+      <c r="T15" s="157"/>
+      <c r="U15" s="157"/>
+      <c r="V15" s="157"/>
+      <c r="W15" s="157"/>
+      <c r="X15" s="157"/>
+      <c r="Y15" s="157"/>
+      <c r="Z15" s="157"/>
+      <c r="AA15" s="158"/>
     </row>
     <row r="16">
-      <c r="A16" s="164" t="s">
-        <v>242</v>
-      </c>
-      <c r="B16" s="153" t="s">
-        <v>243</v>
-      </c>
-      <c r="AA16" s="158"/>
+      <c r="A16" s="166" t="s">
+        <v>246</v>
+      </c>
+      <c r="B16" s="155" t="s">
+        <v>247</v>
+      </c>
+      <c r="AA16" s="160"/>
     </row>
     <row r="17">
-      <c r="A17" s="164" t="s">
+      <c r="A17" s="166" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="153" t="s">
-        <v>244</v>
-      </c>
-      <c r="AA17" s="158"/>
+      <c r="B17" s="155" t="s">
+        <v>248</v>
+      </c>
+      <c r="AA17" s="160"/>
     </row>
     <row r="18">
-      <c r="A18" s="164" t="s">
-        <v>245</v>
-      </c>
-      <c r="B18" s="153" t="s">
-        <v>246</v>
-      </c>
-      <c r="AA18" s="158"/>
+      <c r="A18" s="166" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" s="155" t="s">
+        <v>250</v>
+      </c>
+      <c r="AA18" s="160"/>
     </row>
     <row r="19">
-      <c r="A19" s="165" t="s">
-        <v>247</v>
-      </c>
-      <c r="B19" s="160" t="s">
-        <v>248</v>
-      </c>
-      <c r="C19" s="161"/>
-      <c r="D19" s="161"/>
-      <c r="E19" s="161"/>
-      <c r="F19" s="161"/>
-      <c r="G19" s="161"/>
-      <c r="H19" s="161"/>
-      <c r="I19" s="161"/>
-      <c r="J19" s="161"/>
-      <c r="K19" s="161"/>
-      <c r="L19" s="161"/>
-      <c r="M19" s="161"/>
-      <c r="N19" s="161"/>
-      <c r="O19" s="161"/>
-      <c r="P19" s="161"/>
-      <c r="Q19" s="161"/>
-      <c r="R19" s="161"/>
-      <c r="S19" s="161"/>
-      <c r="T19" s="161"/>
-      <c r="U19" s="161"/>
-      <c r="V19" s="161"/>
-      <c r="W19" s="161"/>
-      <c r="X19" s="161"/>
-      <c r="Y19" s="161"/>
-      <c r="Z19" s="161"/>
-      <c r="AA19" s="162"/>
+      <c r="A19" s="167" t="s">
+        <v>251</v>
+      </c>
+      <c r="B19" s="162" t="s">
+        <v>252</v>
+      </c>
+      <c r="C19" s="163"/>
+      <c r="D19" s="163"/>
+      <c r="E19" s="163"/>
+      <c r="F19" s="163"/>
+      <c r="G19" s="163"/>
+      <c r="H19" s="163"/>
+      <c r="I19" s="163"/>
+      <c r="J19" s="163"/>
+      <c r="K19" s="163"/>
+      <c r="L19" s="163"/>
+      <c r="M19" s="163"/>
+      <c r="N19" s="163"/>
+      <c r="O19" s="163"/>
+      <c r="P19" s="163"/>
+      <c r="Q19" s="163"/>
+      <c r="R19" s="163"/>
+      <c r="S19" s="163"/>
+      <c r="T19" s="163"/>
+      <c r="U19" s="163"/>
+      <c r="V19" s="163"/>
+      <c r="W19" s="163"/>
+      <c r="X19" s="163"/>
+      <c r="Y19" s="163"/>
+      <c r="Z19" s="163"/>
+      <c r="AA19" s="164"/>
     </row>
     <row r="20">
-      <c r="A20" s="153" t="s">
-        <v>249</v>
+      <c r="A20" s="155" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="153" t="s">
-        <v>250</v>
+      <c r="A21" s="155" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="166" t="s">
-        <v>251</v>
+      <c r="A23" s="168" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="166" t="s">
-        <v>252</v>
+      <c r="A24" s="168" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="166" t="s">
-        <v>253</v>
+      <c r="A25" s="168" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>